<commit_message>
Update schedule via dashboard 2026-06-25T14:37:53.083Z
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -652,6 +652,9 @@
     <t>Assistance for Support</t>
   </si>
   <si>
+    <t>Generated on behalf of Ali Raoofi on Thursday, June 25, 2026 9:37:42 AM</t>
+  </si>
+  <si>
     <t>Base Collections in production</t>
   </si>
   <si>
@@ -688,10 +691,6 @@
   <si>
     <t>11/02/26 -
 11/08/26</t>
-  </si>
-  <si>
-    <t>08/03/26 -
-08/09/26</t>
   </si>
   <si>
     <t>List and map - all existing reports and Smartlists</t>
@@ -1091,7 +1090,8 @@
     <t>CIS Go Live - Import Data</t>
   </si>
   <si>
-    <t>Generated on behalf of Ali Raoofi on Thursday, June 25, 2026 9:18:04 AM</t>
+    <t>08/03/26 -
+08/09/26</t>
   </si>
   <si>
     <t>SB-4.6 - Silverblaze Product Guide</t>
@@ -1853,7 +1853,7 @@
     </row>
     <row r="5" spans="1:35" ht="12.75" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>350</v>
+        <v>207</v>
       </c>
     </row>
     <row r="7" spans="1:35" ht="18.75" customHeight="1">
@@ -1905,7 +1905,7 @@
         <v>364</v>
       </c>
       <c r="O9" s="4" t="s">
-        <v>219</v>
+        <v>350</v>
       </c>
       <c r="P9" s="4" t="s">
         <v>93</v>
@@ -1941,10 +1941,10 @@
         <v>83</v>
       </c>
       <c r="AA9" s="4" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AB9" s="4" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AC9" s="4" t="s">
         <v>272</v>
@@ -1994,10 +1994,10 @@
         <v>252</v>
       </c>
       <c r="I10" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J10" s="6">
-        <v>269.4</v>
+        <v>267.9</v>
       </c>
       <c r="K10" s="6">
         <v>247.44</v>
@@ -2101,7 +2101,7 @@
         <v>252</v>
       </c>
       <c r="I11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J11" s="6">
         <v>37.5</v>
@@ -2208,7 +2208,7 @@
         <v>51936</v>
       </c>
       <c r="I12" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J12" s="7">
         <v>19.5</v>
@@ -2850,7 +2850,7 @@
         <v>46248</v>
       </c>
       <c r="I18" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J18" t="s">
         <v>252</v>
@@ -3046,7 +3046,7 @@
         <v>252</v>
       </c>
       <c r="C20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D20" t="s">
         <v>323</v>
@@ -3064,7 +3064,7 @@
         <v>46241</v>
       </c>
       <c r="I20" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J20" s="7">
         <v>0</v>
@@ -3278,7 +3278,7 @@
         <v>46314</v>
       </c>
       <c r="I22" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J22" s="7">
         <v>4</v>
@@ -3492,7 +3492,7 @@
         <v>46213</v>
       </c>
       <c r="I24" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J24" s="7">
         <v>8</v>
@@ -3688,7 +3688,7 @@
         <v>252</v>
       </c>
       <c r="C26" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D26" t="s">
         <v>166</v>
@@ -3706,7 +3706,7 @@
         <v>46752</v>
       </c>
       <c r="I26" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J26" s="7">
         <v>4</v>
@@ -4660,7 +4660,7 @@
         <v>103</v>
       </c>
       <c r="F35" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G35" s="11">
         <v>46101</v>
@@ -4669,7 +4669,7 @@
         <v>46304</v>
       </c>
       <c r="I35" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J35" s="7">
         <v>1</v>
@@ -4883,7 +4883,7 @@
         <v>46304</v>
       </c>
       <c r="I37" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J37" s="7">
         <v>1</v>
@@ -5097,7 +5097,7 @@
         <v>252</v>
       </c>
       <c r="I39" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J39" s="7">
         <v>27.89</v>
@@ -5204,7 +5204,7 @@
         <v>51936</v>
       </c>
       <c r="I40" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J40" s="7">
         <v>7.63</v>
@@ -5834,7 +5834,7 @@
         <v>381</v>
       </c>
       <c r="E46" s="12" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F46" t="s">
         <v>252</v>
@@ -5953,7 +5953,7 @@
         <v>46234</v>
       </c>
       <c r="I47" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J47" s="7">
         <v>20.26</v>
@@ -6274,7 +6274,7 @@
         <v>252</v>
       </c>
       <c r="I50" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J50" s="9">
         <v>50.91</v>
@@ -6381,7 +6381,7 @@
         <v>51936</v>
       </c>
       <c r="I51" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J51" s="7">
         <v>12.5</v>
@@ -7023,7 +7023,7 @@
         <v>46234</v>
       </c>
       <c r="I57" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J57" t="s">
         <v>252</v>
@@ -7237,7 +7237,7 @@
         <v>46387</v>
       </c>
       <c r="I59" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J59" t="s">
         <v>252</v>
@@ -7558,7 +7558,7 @@
         <v>46259</v>
       </c>
       <c r="I62" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J62" t="s">
         <v>252</v>
@@ -7861,7 +7861,7 @@
         <v>252</v>
       </c>
       <c r="C65" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D65" t="s">
         <v>323</v>
@@ -7879,7 +7879,7 @@
         <v>46241</v>
       </c>
       <c r="I65" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J65" s="5" t="s">
         <v>252</v>
@@ -8200,7 +8200,7 @@
         <v>46234</v>
       </c>
       <c r="I68" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J68" s="7">
         <v>29.63</v>
@@ -8628,7 +8628,7 @@
         <v>46308</v>
       </c>
       <c r="I72" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J72" t="s">
         <v>252</v>
@@ -9270,7 +9270,7 @@
         <v>46353</v>
       </c>
       <c r="I78" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J78" t="s">
         <v>252</v>
@@ -10661,7 +10661,7 @@
         <v>46213</v>
       </c>
       <c r="I91" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J91" s="7">
         <v>0.03</v>
@@ -10875,7 +10875,7 @@
         <v>46426</v>
       </c>
       <c r="I93" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J93" t="s">
         <v>252</v>
@@ -11499,7 +11499,7 @@
         <v>252</v>
       </c>
       <c r="C99" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D99" t="s">
         <v>166</v>
@@ -11517,7 +11517,7 @@
         <v>46752</v>
       </c>
       <c r="I99" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J99" s="7">
         <v>1</v>
@@ -12694,7 +12694,7 @@
         <v>46349</v>
       </c>
       <c r="I110" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J110" t="s">
         <v>252</v>
@@ -13764,7 +13764,7 @@
         <v>46164</v>
       </c>
       <c r="I120" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J120" t="s">
         <v>252</v>
@@ -13969,7 +13969,7 @@
         <v>103</v>
       </c>
       <c r="F122" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G122" s="11">
         <v>46101</v>
@@ -13978,7 +13978,7 @@
         <v>46304</v>
       </c>
       <c r="I122" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J122" s="7">
         <v>0.24</v>
@@ -14192,7 +14192,7 @@
         <v>46304</v>
       </c>
       <c r="I124" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J124" s="7">
         <v>0.51</v>
@@ -14406,7 +14406,7 @@
         <v>46248</v>
       </c>
       <c r="I126" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J126" t="s">
         <v>252</v>
@@ -14602,7 +14602,7 @@
         <v>252</v>
       </c>
       <c r="C128" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D128" t="s">
         <v>391</v>
@@ -14620,7 +14620,7 @@
         <v>46237</v>
       </c>
       <c r="I128" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J128" s="7">
         <v>7</v>
@@ -14941,7 +14941,7 @@
         <v>252</v>
       </c>
       <c r="I131" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J131" t="s">
         <v>252</v>
@@ -15048,7 +15048,7 @@
         <v>51936</v>
       </c>
       <c r="I132" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J132" t="s">
         <v>252</v>
@@ -15262,7 +15262,7 @@
         <v>46241</v>
       </c>
       <c r="I134" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J134" t="s">
         <v>252</v>
@@ -15476,7 +15476,7 @@
         <v>252</v>
       </c>
       <c r="I136" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J136" s="7">
         <v>30.48</v>
@@ -15583,7 +15583,7 @@
         <v>51936</v>
       </c>
       <c r="I137" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J137" s="7">
         <v>15</v>
@@ -16225,7 +16225,7 @@
         <v>46234</v>
       </c>
       <c r="I143" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J143" t="s">
         <v>252</v>
@@ -16439,7 +16439,7 @@
         <v>46259</v>
       </c>
       <c r="I145" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J145" s="7">
         <v>10</v>
@@ -17384,7 +17384,7 @@
         <v>252</v>
       </c>
       <c r="C154" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D154" t="s">
         <v>323</v>
@@ -17402,7 +17402,7 @@
         <v>46241</v>
       </c>
       <c r="I154" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J154" t="s">
         <v>252</v>
@@ -17616,7 +17616,7 @@
         <v>46234</v>
       </c>
       <c r="I156" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J156" t="s">
         <v>252</v>
@@ -17937,7 +17937,7 @@
         <v>46353</v>
       </c>
       <c r="I159" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J159" s="7">
         <v>5</v>
@@ -19435,7 +19435,7 @@
         <v>46213</v>
       </c>
       <c r="I173" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J173" t="s">
         <v>252</v>
@@ -19649,7 +19649,7 @@
         <v>46426</v>
       </c>
       <c r="I175" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J175" t="s">
         <v>252</v>
@@ -19863,7 +19863,7 @@
         <v>46349</v>
       </c>
       <c r="I177" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J177" t="s">
         <v>252</v>
@@ -20291,7 +20291,7 @@
         <v>46164</v>
       </c>
       <c r="I181" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J181" t="s">
         <v>252</v>
@@ -20505,7 +20505,7 @@
         <v>46304</v>
       </c>
       <c r="I183" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J183" s="7">
         <v>0.48</v>
@@ -20719,7 +20719,7 @@
         <v>252</v>
       </c>
       <c r="I185" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J185" s="7">
         <v>30.62</v>
@@ -20826,7 +20826,7 @@
         <v>51936</v>
       </c>
       <c r="I186" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J186" s="7">
         <v>15</v>
@@ -21468,7 +21468,7 @@
         <v>46259</v>
       </c>
       <c r="I192" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J192" s="7">
         <v>1</v>
@@ -22413,7 +22413,7 @@
         <v>252</v>
       </c>
       <c r="C201" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D201" t="s">
         <v>323</v>
@@ -22431,7 +22431,7 @@
         <v>46241</v>
       </c>
       <c r="I201" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J201" s="7">
         <v>0.02</v>
@@ -22752,7 +22752,7 @@
         <v>46234</v>
       </c>
       <c r="I204" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J204" s="7">
         <v>10</v>
@@ -23073,7 +23073,7 @@
         <v>46248</v>
       </c>
       <c r="I207" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J207" s="7">
         <v>0.86</v>
@@ -23376,7 +23376,7 @@
         <v>252</v>
       </c>
       <c r="C210" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D210" t="s">
         <v>391</v>
@@ -23394,7 +23394,7 @@
         <v>46237</v>
       </c>
       <c r="I210" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J210" s="7">
         <v>3.75</v>
@@ -23608,10 +23608,10 @@
         <v>252</v>
       </c>
       <c r="I212" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J212" s="6">
-        <v>37.5</v>
+        <v>38.5</v>
       </c>
       <c r="K212" s="6">
         <v>33.5</v>
@@ -23715,7 +23715,7 @@
         <v>51936</v>
       </c>
       <c r="I213" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J213" s="7">
         <v>13.5</v>
@@ -24357,7 +24357,7 @@
         <v>46387</v>
       </c>
       <c r="I219" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J219" t="s">
         <v>252</v>
@@ -24678,10 +24678,10 @@
         <v>46259</v>
       </c>
       <c r="I222" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J222" s="7">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="K222" s="7">
         <v>20</v>
@@ -24895,7 +24895,7 @@
         <v>252</v>
       </c>
       <c r="J224" s="7">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="K224" t="s">
         <v>252</v>
@@ -25109,7 +25109,7 @@
         <v>252</v>
       </c>
       <c r="J226" s="7">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="K226" t="s">
         <v>252</v>
@@ -25944,7 +25944,7 @@
         <v>252</v>
       </c>
       <c r="C234" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D234" t="s">
         <v>323</v>
@@ -25962,7 +25962,7 @@
         <v>46241</v>
       </c>
       <c r="I234" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J234" t="s">
         <v>252</v>
@@ -26176,10 +26176,10 @@
         <v>46205</v>
       </c>
       <c r="I236" t="s">
-        <v>212</v>
-      </c>
-      <c r="J236" s="7">
-        <v>5</v>
+        <v>213</v>
+      </c>
+      <c r="J236" t="s">
+        <v>252</v>
       </c>
       <c r="K236" t="s">
         <v>252</v>
@@ -26285,8 +26285,8 @@
       <c r="I237" t="s">
         <v>252</v>
       </c>
-      <c r="J237" s="7">
-        <v>5</v>
+      <c r="J237" t="s">
+        <v>252</v>
       </c>
       <c r="K237" t="s">
         <v>252</v>
@@ -26390,10 +26390,10 @@
         <v>46241</v>
       </c>
       <c r="I238" t="s">
-        <v>212</v>
-      </c>
-      <c r="J238" s="7">
-        <v>2</v>
+        <v>213</v>
+      </c>
+      <c r="J238" t="s">
+        <v>252</v>
       </c>
       <c r="K238" s="7">
         <v>1</v>
@@ -26499,8 +26499,8 @@
       <c r="I239" t="s">
         <v>252</v>
       </c>
-      <c r="J239" s="7">
-        <v>2</v>
+      <c r="J239" t="s">
+        <v>252</v>
       </c>
       <c r="K239" s="7">
         <v>1</v>
@@ -26604,10 +26604,10 @@
         <v>46308</v>
       </c>
       <c r="I240" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J240" s="7">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K240" t="s">
         <v>252</v>
@@ -26714,7 +26714,7 @@
         <v>252</v>
       </c>
       <c r="J241" s="7">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K241" t="s">
         <v>252</v>
@@ -26818,7 +26818,7 @@
         <v>46426</v>
       </c>
       <c r="I242" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J242" s="7">
         <v>1</v>
@@ -27656,7 +27656,7 @@
         <v>252</v>
       </c>
       <c r="C250" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D250" t="s">
         <v>166</v>
@@ -27674,7 +27674,7 @@
         <v>46752</v>
       </c>
       <c r="I250" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J250" s="7">
         <v>3</v>
@@ -28530,10 +28530,10 @@
         <v>252</v>
       </c>
       <c r="I258" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J258" s="6">
-        <v>39.5</v>
+        <v>37</v>
       </c>
       <c r="K258" s="7">
         <v>13.5</v>
@@ -28637,10 +28637,10 @@
         <v>51936</v>
       </c>
       <c r="I259" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J259" s="7">
-        <v>15</v>
+        <v>12.5</v>
       </c>
       <c r="K259" s="7">
         <v>7.5</v>
@@ -28854,7 +28854,7 @@
         <v>252</v>
       </c>
       <c r="J261" s="7">
-        <v>7.5</v>
+        <v>5</v>
       </c>
       <c r="K261" s="7">
         <v>7.5</v>
@@ -29261,7 +29261,7 @@
         <v>252</v>
       </c>
       <c r="C265" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D265" t="s">
         <v>323</v>
@@ -29279,7 +29279,7 @@
         <v>46241</v>
       </c>
       <c r="I265" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J265" s="5" t="s">
         <v>252</v>
@@ -29493,7 +29493,7 @@
         <v>46241</v>
       </c>
       <c r="I267" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J267" t="s">
         <v>252</v>
@@ -29796,7 +29796,7 @@
         <v>252</v>
       </c>
       <c r="C270" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D270" t="s">
         <v>166</v>
@@ -29814,7 +29814,7 @@
         <v>46752</v>
       </c>
       <c r="I270" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J270" s="6">
         <v>24.5</v>
@@ -30979,7 +30979,7 @@
         <v>166</v>
       </c>
       <c r="E281" s="12" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F281" t="s">
         <v>252</v>
@@ -31514,7 +31514,7 @@
         <v>166</v>
       </c>
       <c r="E286" s="12" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F286" t="s">
         <v>252</v>
@@ -33131,7 +33131,7 @@
         <v>252</v>
       </c>
       <c r="I301" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J301" s="7">
         <v>15</v>
@@ -33238,7 +33238,7 @@
         <v>51936</v>
       </c>
       <c r="I302" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J302" s="7">
         <v>12.5</v>
@@ -33862,7 +33862,7 @@
         <v>252</v>
       </c>
       <c r="C308" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D308" t="s">
         <v>166</v>
@@ -33880,7 +33880,7 @@
         <v>46752</v>
       </c>
       <c r="I308" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J308" s="7">
         <v>2.5</v>
@@ -34510,7 +34510,7 @@
         <v>166</v>
       </c>
       <c r="E314" s="12" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F314" t="s">
         <v>252</v>
@@ -35592,7 +35592,7 @@
         <v>46349</v>
       </c>
       <c r="I324" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J324" t="s">
         <v>252</v>
@@ -35806,31 +35806,31 @@
         <v>252</v>
       </c>
       <c r="I326" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J326" s="6">
-        <v>94.27</v>
+        <v>106.98</v>
       </c>
       <c r="K326" s="9">
-        <v>118.71</v>
+        <v>115.65</v>
       </c>
       <c r="L326" s="6">
-        <v>105.23</v>
+        <v>106.17</v>
       </c>
       <c r="M326" s="7">
-        <v>68.09</v>
-      </c>
-      <c r="N326" s="9">
-        <v>121.59</v>
+        <v>69.06</v>
+      </c>
+      <c r="N326" s="7">
+        <v>102.56</v>
       </c>
       <c r="O326" s="6">
-        <v>107.09</v>
+        <v>104.86</v>
       </c>
       <c r="P326" s="6">
-        <v>104.59</v>
+        <v>102.36</v>
       </c>
       <c r="Q326" s="7">
-        <v>82.09</v>
+        <v>79.86</v>
       </c>
       <c r="R326" s="7">
         <v>39.66</v>
@@ -35913,31 +35913,31 @@
         <v>252</v>
       </c>
       <c r="I327" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J327" s="7">
-        <v>25.99</v>
+        <v>35.5</v>
       </c>
       <c r="K327" s="6">
-        <v>40.96</v>
+        <v>34.7</v>
       </c>
       <c r="L327" s="7">
-        <v>14.86</v>
+        <v>12.6</v>
       </c>
       <c r="M327" s="7">
-        <v>13.73</v>
+        <v>11.5</v>
       </c>
       <c r="N327" s="7">
-        <v>34.73</v>
+        <v>37.5</v>
       </c>
       <c r="O327" s="9">
-        <v>44.73</v>
+        <v>42.5</v>
       </c>
       <c r="P327" s="7">
-        <v>14.73</v>
+        <v>12.5</v>
       </c>
       <c r="Q327" s="7">
-        <v>29.73</v>
+        <v>27.5</v>
       </c>
       <c r="R327" s="7">
         <v>9.73</v>
@@ -36020,10 +36020,10 @@
         <v>51936</v>
       </c>
       <c r="I328" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J328" s="7">
-        <v>15</v>
+        <v>12.5</v>
       </c>
       <c r="K328" s="7">
         <v>7.5</v>
@@ -36237,7 +36237,7 @@
         <v>252</v>
       </c>
       <c r="J330" s="7">
-        <v>7.5</v>
+        <v>5</v>
       </c>
       <c r="K330" s="7">
         <v>7.5</v>
@@ -36662,10 +36662,10 @@
         <v>46213</v>
       </c>
       <c r="I334" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J334" s="7">
-        <v>5.5</v>
+        <v>10</v>
       </c>
       <c r="K334" s="7">
         <v>5.5</v>
@@ -36772,7 +36772,7 @@
         <v>252</v>
       </c>
       <c r="J335" s="7">
-        <v>5.5</v>
+        <v>10</v>
       </c>
       <c r="K335" s="7">
         <v>5.5</v>
@@ -36876,13 +36876,13 @@
         <v>46234</v>
       </c>
       <c r="I336" t="s">
-        <v>212</v>
-      </c>
-      <c r="J336" t="s">
-        <v>252</v>
-      </c>
-      <c r="K336" s="7">
+        <v>213</v>
+      </c>
+      <c r="J336" s="7">
         <v>4</v>
+      </c>
+      <c r="K336" t="s">
+        <v>252</v>
       </c>
       <c r="L336" t="s">
         <v>252</v>
@@ -36985,11 +36985,11 @@
       <c r="I337" t="s">
         <v>252</v>
       </c>
-      <c r="J337" t="s">
-        <v>252</v>
-      </c>
-      <c r="K337" s="7">
+      <c r="J337" s="7">
         <v>4</v>
+      </c>
+      <c r="K337" t="s">
+        <v>252</v>
       </c>
       <c r="L337" t="s">
         <v>252</v>
@@ -37090,10 +37090,10 @@
         <v>46255</v>
       </c>
       <c r="I338" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J338" s="7">
-        <v>2.43</v>
+        <v>3</v>
       </c>
       <c r="K338" s="6">
         <v>20</v>
@@ -37307,7 +37307,7 @@
         <v>252</v>
       </c>
       <c r="J340" s="7">
-        <v>1.43</v>
+        <v>2</v>
       </c>
       <c r="K340" t="s">
         <v>252</v>
@@ -37931,10 +37931,10 @@
         <v>82</v>
       </c>
       <c r="D346" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E346" s="10" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F346" t="s">
         <v>235</v>
@@ -37946,31 +37946,31 @@
         <v>46454</v>
       </c>
       <c r="I346" t="s">
-        <v>212</v>
-      </c>
-      <c r="J346" s="7">
-        <v>1.34</v>
-      </c>
-      <c r="K346" s="7">
-        <v>2.23</v>
-      </c>
-      <c r="L346" s="7">
-        <v>2.23</v>
-      </c>
-      <c r="M346" s="7">
-        <v>2.23</v>
-      </c>
-      <c r="N346" s="7">
-        <v>2.23</v>
-      </c>
-      <c r="O346" s="7">
-        <v>2.23</v>
-      </c>
-      <c r="P346" s="7">
-        <v>2.23</v>
-      </c>
-      <c r="Q346" s="7">
-        <v>2.23</v>
+        <v>213</v>
+      </c>
+      <c r="J346" t="s">
+        <v>252</v>
+      </c>
+      <c r="K346" t="s">
+        <v>252</v>
+      </c>
+      <c r="L346" t="s">
+        <v>252</v>
+      </c>
+      <c r="M346" t="s">
+        <v>252</v>
+      </c>
+      <c r="N346" t="s">
+        <v>252</v>
+      </c>
+      <c r="O346" t="s">
+        <v>252</v>
+      </c>
+      <c r="P346" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q346" t="s">
+        <v>252</v>
       </c>
       <c r="R346" s="7">
         <v>2.23</v>
@@ -38038,7 +38038,7 @@
         <v>252</v>
       </c>
       <c r="D347" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E347" s="12" t="s">
         <v>341</v>
@@ -38055,29 +38055,29 @@
       <c r="I347" t="s">
         <v>252</v>
       </c>
-      <c r="J347" s="7">
-        <v>1.34</v>
-      </c>
-      <c r="K347" s="7">
-        <v>2.23</v>
-      </c>
-      <c r="L347" s="7">
-        <v>2.23</v>
-      </c>
-      <c r="M347" s="7">
-        <v>2.23</v>
-      </c>
-      <c r="N347" s="7">
-        <v>2.23</v>
-      </c>
-      <c r="O347" s="7">
-        <v>2.23</v>
-      </c>
-      <c r="P347" s="7">
-        <v>2.23</v>
-      </c>
-      <c r="Q347" s="7">
-        <v>2.23</v>
+      <c r="J347" t="s">
+        <v>252</v>
+      </c>
+      <c r="K347" t="s">
+        <v>252</v>
+      </c>
+      <c r="L347" t="s">
+        <v>252</v>
+      </c>
+      <c r="M347" t="s">
+        <v>252</v>
+      </c>
+      <c r="N347" t="s">
+        <v>252</v>
+      </c>
+      <c r="O347" t="s">
+        <v>252</v>
+      </c>
+      <c r="P347" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q347" t="s">
+        <v>252</v>
       </c>
       <c r="R347" s="7">
         <v>2.23</v>
@@ -38145,7 +38145,7 @@
         <v>252</v>
       </c>
       <c r="D348" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E348" s="12" t="s">
         <v>162</v>
@@ -38252,7 +38252,7 @@
         <v>252</v>
       </c>
       <c r="D349" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E349" s="12" t="s">
         <v>369</v>
@@ -38359,7 +38359,7 @@
         <v>252</v>
       </c>
       <c r="D350" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E350" s="12" t="s">
         <v>144</v>
@@ -38466,7 +38466,7 @@
         <v>252</v>
       </c>
       <c r="D351" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E351" s="12" t="s">
         <v>126</v>
@@ -38573,7 +38573,7 @@
         <v>252</v>
       </c>
       <c r="D352" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E352" s="12" t="s">
         <v>363</v>
@@ -38680,7 +38680,7 @@
         <v>252</v>
       </c>
       <c r="D353" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E353" s="12" t="s">
         <v>27</v>
@@ -38787,10 +38787,10 @@
         <v>252</v>
       </c>
       <c r="D354" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E354" s="12" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F354" t="s">
         <v>252</v>
@@ -38894,7 +38894,7 @@
         <v>252</v>
       </c>
       <c r="D355" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E355" s="12" t="s">
         <v>266</v>
@@ -39016,16 +39016,16 @@
         <v>46511</v>
       </c>
       <c r="I356" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J356" s="7">
-        <v>1.73</v>
+        <v>2</v>
       </c>
       <c r="K356" s="7">
-        <v>1.73</v>
+        <v>1.7</v>
       </c>
       <c r="L356" s="7">
-        <v>1.73</v>
+        <v>1.7</v>
       </c>
       <c r="M356" t="s">
         <v>252</v>
@@ -39126,13 +39126,13 @@
         <v>252</v>
       </c>
       <c r="J357" s="7">
-        <v>1.73</v>
+        <v>2</v>
       </c>
       <c r="K357" s="7">
-        <v>1.73</v>
+        <v>1.7</v>
       </c>
       <c r="L357" s="7">
-        <v>1.73</v>
+        <v>1.7</v>
       </c>
       <c r="M357" t="s">
         <v>252</v>
@@ -39230,10 +39230,10 @@
         <v>46283</v>
       </c>
       <c r="I358" t="s">
-        <v>212</v>
-      </c>
-      <c r="J358" t="s">
-        <v>252</v>
+        <v>213</v>
+      </c>
+      <c r="J358" s="7">
+        <v>4</v>
       </c>
       <c r="K358" t="s">
         <v>252</v>
@@ -39245,7 +39245,7 @@
         <v>252</v>
       </c>
       <c r="N358" s="7">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="O358" s="7">
         <v>5</v>
@@ -39331,7 +39331,7 @@
         <v>252</v>
       </c>
       <c r="G359" s="11">
-        <v>46230</v>
+        <v>46202</v>
       </c>
       <c r="H359" s="11">
         <v>46234</v>
@@ -39339,8 +39339,8 @@
       <c r="I359" t="s">
         <v>252</v>
       </c>
-      <c r="J359" t="s">
-        <v>252</v>
+      <c r="J359" s="7">
+        <v>4</v>
       </c>
       <c r="K359" t="s">
         <v>252</v>
@@ -39352,7 +39352,7 @@
         <v>252</v>
       </c>
       <c r="N359" s="7">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="O359" t="s">
         <v>252</v>
@@ -39551,22 +39551,22 @@
         <v>252</v>
       </c>
       <c r="I361" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J361" s="7">
-        <v>23.35</v>
+        <v>26.55</v>
       </c>
       <c r="K361" s="6">
-        <v>21.75</v>
+        <v>24.95</v>
       </c>
       <c r="L361" s="6">
-        <v>34.44</v>
+        <v>37.64</v>
       </c>
       <c r="M361" s="7">
-        <v>32.43</v>
-      </c>
-      <c r="N361" s="9">
-        <v>57.43</v>
+        <v>35.63</v>
+      </c>
+      <c r="N361" s="7">
+        <v>35.63</v>
       </c>
       <c r="O361" s="9">
         <v>44.93</v>
@@ -39658,7 +39658,7 @@
         <v>51936</v>
       </c>
       <c r="I362" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J362" s="7">
         <v>15</v>
@@ -40300,7 +40300,7 @@
         <v>46213</v>
       </c>
       <c r="I368" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J368" s="7">
         <v>1.25</v>
@@ -40514,7 +40514,7 @@
         <v>46255</v>
       </c>
       <c r="I370" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J370" s="7">
         <v>5</v>
@@ -41355,10 +41355,10 @@
         <v>82</v>
       </c>
       <c r="D378" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E378" s="10" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F378" t="s">
         <v>235</v>
@@ -41370,7 +41370,7 @@
         <v>46454</v>
       </c>
       <c r="I378" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J378" t="s">
         <v>252</v>
@@ -41462,7 +41462,7 @@
         <v>252</v>
       </c>
       <c r="D379" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E379" s="12" t="s">
         <v>341</v>
@@ -41569,7 +41569,7 @@
         <v>252</v>
       </c>
       <c r="D380" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E380" s="12" t="s">
         <v>133</v>
@@ -41676,7 +41676,7 @@
         <v>252</v>
       </c>
       <c r="D381" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E381" s="12" t="s">
         <v>5</v>
@@ -41783,7 +41783,7 @@
         <v>252</v>
       </c>
       <c r="D382" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E382" s="12" t="s">
         <v>124</v>
@@ -41890,7 +41890,7 @@
         <v>252</v>
       </c>
       <c r="D383" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E383" s="12" t="s">
         <v>51</v>
@@ -41997,7 +41997,7 @@
         <v>252</v>
       </c>
       <c r="D384" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E384" s="12" t="s">
         <v>320</v>
@@ -42104,7 +42104,7 @@
         <v>252</v>
       </c>
       <c r="D385" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E385" s="12" t="s">
         <v>162</v>
@@ -42211,7 +42211,7 @@
         <v>252</v>
       </c>
       <c r="D386" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E386" s="12" t="s">
         <v>263</v>
@@ -42318,7 +42318,7 @@
         <v>252</v>
       </c>
       <c r="D387" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E387" s="12" t="s">
         <v>342</v>
@@ -42425,7 +42425,7 @@
         <v>252</v>
       </c>
       <c r="D388" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E388" s="12" t="s">
         <v>369</v>
@@ -42532,7 +42532,7 @@
         <v>252</v>
       </c>
       <c r="D389" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E389" s="12" t="s">
         <v>144</v>
@@ -42639,7 +42639,7 @@
         <v>252</v>
       </c>
       <c r="D390" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E390" s="12" t="s">
         <v>126</v>
@@ -42746,7 +42746,7 @@
         <v>252</v>
       </c>
       <c r="D391" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E391" s="12" t="s">
         <v>363</v>
@@ -42853,7 +42853,7 @@
         <v>252</v>
       </c>
       <c r="D392" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E392" s="12" t="s">
         <v>27</v>
@@ -42960,10 +42960,10 @@
         <v>252</v>
       </c>
       <c r="D393" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E393" s="12" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F393" t="s">
         <v>252</v>
@@ -43067,7 +43067,7 @@
         <v>252</v>
       </c>
       <c r="D394" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E394" s="12" t="s">
         <v>266</v>
@@ -43189,7 +43189,7 @@
         <v>46511</v>
       </c>
       <c r="I395" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J395" s="7">
         <v>2.1</v>
@@ -43403,22 +43403,22 @@
         <v>46283</v>
       </c>
       <c r="I397" t="s">
-        <v>212</v>
-      </c>
-      <c r="J397" t="s">
-        <v>252</v>
-      </c>
-      <c r="K397" t="s">
-        <v>252</v>
-      </c>
-      <c r="L397" t="s">
-        <v>252</v>
-      </c>
-      <c r="M397" t="s">
-        <v>252</v>
+        <v>213</v>
+      </c>
+      <c r="J397" s="7">
+        <v>3.2</v>
+      </c>
+      <c r="K397" s="7">
+        <v>3.2</v>
+      </c>
+      <c r="L397" s="7">
+        <v>3.2</v>
+      </c>
+      <c r="M397" s="7">
+        <v>3.2</v>
       </c>
       <c r="N397" s="7">
-        <v>25</v>
+        <v>3.2</v>
       </c>
       <c r="O397" s="7">
         <v>5</v>
@@ -43504,7 +43504,7 @@
         <v>252</v>
       </c>
       <c r="G398" s="11">
-        <v>46230</v>
+        <v>46202</v>
       </c>
       <c r="H398" s="11">
         <v>46234</v>
@@ -43512,20 +43512,20 @@
       <c r="I398" t="s">
         <v>252</v>
       </c>
-      <c r="J398" t="s">
-        <v>252</v>
-      </c>
-      <c r="K398" t="s">
-        <v>252</v>
-      </c>
-      <c r="L398" t="s">
-        <v>252</v>
-      </c>
-      <c r="M398" t="s">
-        <v>252</v>
+      <c r="J398" s="7">
+        <v>3.2</v>
+      </c>
+      <c r="K398" s="7">
+        <v>3.2</v>
+      </c>
+      <c r="L398" s="7">
+        <v>3.2</v>
+      </c>
+      <c r="M398" s="7">
+        <v>3.2</v>
       </c>
       <c r="N398" s="7">
-        <v>25</v>
+        <v>3.2</v>
       </c>
       <c r="O398" t="s">
         <v>252</v>
@@ -43724,7 +43724,7 @@
         <v>252</v>
       </c>
       <c r="I400" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J400" s="9">
         <v>44.93</v>
@@ -43831,7 +43831,7 @@
         <v>51936</v>
       </c>
       <c r="I401" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J401" s="7">
         <v>25.5</v>
@@ -44473,7 +44473,7 @@
         <v>46248</v>
       </c>
       <c r="I407" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J407" t="s">
         <v>252</v>
@@ -44687,7 +44687,7 @@
         <v>46259</v>
       </c>
       <c r="I409" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J409" t="s">
         <v>252</v>
@@ -44901,7 +44901,7 @@
         <v>46213</v>
       </c>
       <c r="I411" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J411" t="s">
         <v>252</v>
@@ -45100,10 +45100,10 @@
         <v>82</v>
       </c>
       <c r="D413" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E413" s="10" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F413" t="s">
         <v>235</v>
@@ -45115,7 +45115,7 @@
         <v>46454</v>
       </c>
       <c r="I413" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J413" s="7">
         <v>6.03</v>
@@ -45207,7 +45207,7 @@
         <v>252</v>
       </c>
       <c r="D414" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E414" s="12" t="s">
         <v>341</v>
@@ -45314,7 +45314,7 @@
         <v>252</v>
       </c>
       <c r="D415" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E415" s="12" t="s">
         <v>336</v>
@@ -45421,7 +45421,7 @@
         <v>252</v>
       </c>
       <c r="D416" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E416" s="12" t="s">
         <v>332</v>
@@ -45528,7 +45528,7 @@
         <v>252</v>
       </c>
       <c r="D417" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E417" s="12" t="s">
         <v>133</v>
@@ -45635,7 +45635,7 @@
         <v>252</v>
       </c>
       <c r="D418" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E418" s="12" t="s">
         <v>5</v>
@@ -45742,7 +45742,7 @@
         <v>252</v>
       </c>
       <c r="D419" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E419" s="12" t="s">
         <v>124</v>
@@ -45849,7 +45849,7 @@
         <v>252</v>
       </c>
       <c r="D420" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E420" s="12" t="s">
         <v>51</v>
@@ -45956,7 +45956,7 @@
         <v>252</v>
       </c>
       <c r="D421" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E421" s="12" t="s">
         <v>320</v>
@@ -46063,7 +46063,7 @@
         <v>252</v>
       </c>
       <c r="D422" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E422" s="12" t="s">
         <v>162</v>
@@ -46170,7 +46170,7 @@
         <v>252</v>
       </c>
       <c r="D423" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E423" s="12" t="s">
         <v>263</v>
@@ -46277,7 +46277,7 @@
         <v>252</v>
       </c>
       <c r="D424" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E424" s="12" t="s">
         <v>342</v>
@@ -46384,7 +46384,7 @@
         <v>252</v>
       </c>
       <c r="D425" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E425" s="12" t="s">
         <v>369</v>
@@ -46491,7 +46491,7 @@
         <v>252</v>
       </c>
       <c r="D426" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E426" s="12" t="s">
         <v>144</v>
@@ -46598,7 +46598,7 @@
         <v>252</v>
       </c>
       <c r="D427" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E427" s="12" t="s">
         <v>126</v>
@@ -46705,7 +46705,7 @@
         <v>252</v>
       </c>
       <c r="D428" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E428" s="12" t="s">
         <v>363</v>
@@ -46812,7 +46812,7 @@
         <v>252</v>
       </c>
       <c r="D429" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E429" s="12" t="s">
         <v>27</v>
@@ -46919,10 +46919,10 @@
         <v>252</v>
       </c>
       <c r="D430" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E430" s="12" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F430" t="s">
         <v>252</v>
@@ -47026,7 +47026,7 @@
         <v>252</v>
       </c>
       <c r="D431" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E431" s="12" t="s">
         <v>266</v>
@@ -47148,7 +47148,7 @@
         <v>46511</v>
       </c>
       <c r="I432" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J432" s="7">
         <v>13.4</v>
@@ -54210,10 +54210,10 @@
         <v>252</v>
       </c>
       <c r="I498" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J498" s="6">
-        <v>114.08</v>
+        <v>119.08</v>
       </c>
       <c r="K498" s="6">
         <v>66.23</v>
@@ -54317,10 +54317,10 @@
         <v>252</v>
       </c>
       <c r="I499" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J499" s="7">
-        <v>22.39</v>
+        <v>27.39</v>
       </c>
       <c r="K499" s="7">
         <v>8.53</v>
@@ -54424,7 +54424,7 @@
         <v>51936</v>
       </c>
       <c r="I500" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J500" s="7">
         <v>15</v>
@@ -55066,7 +55066,7 @@
         <v>46259</v>
       </c>
       <c r="I506" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J506" s="7">
         <v>0.03</v>
@@ -55369,7 +55369,7 @@
         <v>252</v>
       </c>
       <c r="C509" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D509" t="s">
         <v>323</v>
@@ -55387,7 +55387,7 @@
         <v>46241</v>
       </c>
       <c r="I509" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J509" s="7">
         <v>0.02</v>
@@ -55601,10 +55601,10 @@
         <v>46205</v>
       </c>
       <c r="I511" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J511" s="7">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="K511" t="s">
         <v>252</v>
@@ -55711,7 +55711,7 @@
         <v>252</v>
       </c>
       <c r="J512" s="7">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="K512" t="s">
         <v>252</v>
@@ -55815,7 +55815,7 @@
         <v>46308</v>
       </c>
       <c r="I513" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J513" s="7">
         <v>0.35</v>
@@ -56243,7 +56243,7 @@
         <v>46426</v>
       </c>
       <c r="I517" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J517" t="s">
         <v>252</v>
@@ -56653,7 +56653,7 @@
         <v>252</v>
       </c>
       <c r="C521" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D521" t="s">
         <v>166</v>
@@ -56671,7 +56671,7 @@
         <v>46752</v>
       </c>
       <c r="I521" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J521" s="7">
         <v>3</v>
@@ -57420,7 +57420,7 @@
         <v>252</v>
       </c>
       <c r="I528" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J528" s="7">
         <v>20.19</v>
@@ -57527,7 +57527,7 @@
         <v>51936</v>
       </c>
       <c r="I529" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J529" s="7">
         <v>15</v>
@@ -58169,7 +58169,7 @@
         <v>46387</v>
       </c>
       <c r="I535" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J535" t="s">
         <v>252</v>
@@ -58383,7 +58383,7 @@
         <v>46387</v>
       </c>
       <c r="I537" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J537" t="s">
         <v>252</v>
@@ -58597,7 +58597,7 @@
         <v>46387</v>
       </c>
       <c r="I539" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J539" t="s">
         <v>252</v>
@@ -58811,7 +58811,7 @@
         <v>45443</v>
       </c>
       <c r="I541" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J541" t="s">
         <v>252</v>
@@ -59025,7 +59025,7 @@
         <v>46022</v>
       </c>
       <c r="I543" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J543" t="s">
         <v>252</v>
@@ -59239,7 +59239,7 @@
         <v>46387</v>
       </c>
       <c r="I545" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J545" s="5" t="s">
         <v>252</v>
@@ -59453,7 +59453,7 @@
         <v>46387</v>
       </c>
       <c r="I547" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J547" t="s">
         <v>252</v>
@@ -59667,7 +59667,7 @@
         <v>46387</v>
       </c>
       <c r="I549" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J549" t="s">
         <v>252</v>
@@ -59881,7 +59881,7 @@
         <v>46353</v>
       </c>
       <c r="I551" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J551" s="7">
         <v>1.44</v>
@@ -60737,7 +60737,7 @@
         <v>46426</v>
       </c>
       <c r="I559" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J559" s="7">
         <v>3.75</v>
@@ -60951,7 +60951,7 @@
         <v>47003</v>
       </c>
       <c r="I561" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J561" t="s">
         <v>252</v>
@@ -61165,7 +61165,7 @@
         <v>47003</v>
       </c>
       <c r="I563" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J563" t="s">
         <v>252</v>
@@ -61379,7 +61379,7 @@
         <v>46387</v>
       </c>
       <c r="I565" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J565" t="s">
         <v>252</v>
@@ -61593,7 +61593,7 @@
         <v>46387</v>
       </c>
       <c r="I567" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J567" t="s">
         <v>252</v>
@@ -61807,7 +61807,7 @@
         <v>46387</v>
       </c>
       <c r="I569" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J569" t="s">
         <v>252</v>
@@ -62003,7 +62003,7 @@
         <v>252</v>
       </c>
       <c r="C571" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D571" t="s">
         <v>108</v>
@@ -62021,7 +62021,7 @@
         <v>46387</v>
       </c>
       <c r="I571" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J571" t="s">
         <v>252</v>
@@ -62235,7 +62235,7 @@
         <v>252</v>
       </c>
       <c r="I573" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J573" s="7">
         <v>9.65</v>
@@ -62342,7 +62342,7 @@
         <v>51936</v>
       </c>
       <c r="I574" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J574" s="7">
         <v>7.5</v>
@@ -62877,7 +62877,7 @@
         <v>46259</v>
       </c>
       <c r="I579" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J579" t="s">
         <v>252</v>
@@ -63091,7 +63091,7 @@
         <v>46308</v>
       </c>
       <c r="I581" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J581" s="7">
         <v>0.35</v>
@@ -63412,7 +63412,7 @@
         <v>46426</v>
       </c>
       <c r="I584" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J584" s="7">
         <v>1.8</v>
@@ -63733,7 +63733,7 @@
         <v>252</v>
       </c>
       <c r="I587" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J587" s="7">
         <v>17.74</v>
@@ -63840,7 +63840,7 @@
         <v>51936</v>
       </c>
       <c r="I588" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J588" s="7">
         <v>11.68</v>
@@ -64482,7 +64482,7 @@
         <v>46387</v>
       </c>
       <c r="I594" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J594" t="s">
         <v>252</v>
@@ -64696,7 +64696,7 @@
         <v>46387</v>
       </c>
       <c r="I596" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J596" t="s">
         <v>252</v>
@@ -64910,7 +64910,7 @@
         <v>46387</v>
       </c>
       <c r="I598" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J598" t="s">
         <v>252</v>
@@ -65124,7 +65124,7 @@
         <v>45443</v>
       </c>
       <c r="I600" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J600" t="s">
         <v>252</v>
@@ -65338,7 +65338,7 @@
         <v>46022</v>
       </c>
       <c r="I602" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J602" t="s">
         <v>252</v>
@@ -65552,7 +65552,7 @@
         <v>46387</v>
       </c>
       <c r="I604" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J604" s="5" t="s">
         <v>252</v>
@@ -65766,7 +65766,7 @@
         <v>46387</v>
       </c>
       <c r="I606" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J606" t="s">
         <v>252</v>
@@ -65980,7 +65980,7 @@
         <v>46387</v>
       </c>
       <c r="I608" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J608" t="s">
         <v>252</v>
@@ -66194,7 +66194,7 @@
         <v>46259</v>
       </c>
       <c r="I610" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J610" t="s">
         <v>252</v>
@@ -66408,7 +66408,7 @@
         <v>46308</v>
       </c>
       <c r="I612" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J612" s="7">
         <v>6.06</v>
@@ -66836,7 +66836,7 @@
         <v>46426</v>
       </c>
       <c r="I616" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J616" t="s">
         <v>252</v>
@@ -67157,7 +67157,7 @@
         <v>47003</v>
       </c>
       <c r="I619" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J619" t="s">
         <v>252</v>
@@ -67371,7 +67371,7 @@
         <v>47003</v>
       </c>
       <c r="I621" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J621" t="s">
         <v>252</v>
@@ -67585,7 +67585,7 @@
         <v>46387</v>
       </c>
       <c r="I623" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J623" t="s">
         <v>252</v>
@@ -67799,7 +67799,7 @@
         <v>46387</v>
       </c>
       <c r="I625" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J625" t="s">
         <v>252</v>
@@ -68013,7 +68013,7 @@
         <v>46387</v>
       </c>
       <c r="I627" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J627" t="s">
         <v>252</v>
@@ -68209,7 +68209,7 @@
         <v>252</v>
       </c>
       <c r="C629" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D629" t="s">
         <v>108</v>
@@ -68227,7 +68227,7 @@
         <v>46387</v>
       </c>
       <c r="I629" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J629" t="s">
         <v>252</v>
@@ -68420,7 +68420,7 @@
         <v>278</v>
       </c>
       <c r="B631" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C631" t="s">
         <v>252</v>
@@ -68441,7 +68441,7 @@
         <v>252</v>
       </c>
       <c r="I631" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J631" s="6">
         <v>33.57</v>
@@ -68548,7 +68548,7 @@
         <v>51936</v>
       </c>
       <c r="I632" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J632" s="7">
         <v>15</v>
@@ -69190,7 +69190,7 @@
         <v>46387</v>
       </c>
       <c r="I638" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J638" t="s">
         <v>252</v>
@@ -69404,7 +69404,7 @@
         <v>46387</v>
       </c>
       <c r="I640" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J640" t="s">
         <v>252</v>
@@ -69618,7 +69618,7 @@
         <v>46387</v>
       </c>
       <c r="I642" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J642" t="s">
         <v>252</v>
@@ -69832,7 +69832,7 @@
         <v>45443</v>
       </c>
       <c r="I644" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J644" t="s">
         <v>252</v>
@@ -70046,7 +70046,7 @@
         <v>46022</v>
       </c>
       <c r="I646" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J646" t="s">
         <v>252</v>
@@ -70260,7 +70260,7 @@
         <v>46387</v>
       </c>
       <c r="I648" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J648" t="s">
         <v>252</v>
@@ -70474,7 +70474,7 @@
         <v>46387</v>
       </c>
       <c r="I650" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J650" t="s">
         <v>252</v>
@@ -70688,7 +70688,7 @@
         <v>46387</v>
       </c>
       <c r="I652" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J652" t="s">
         <v>252</v>
@@ -70902,7 +70902,7 @@
         <v>46259</v>
       </c>
       <c r="I654" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J654" s="7">
         <v>0.2</v>
@@ -71205,7 +71205,7 @@
         <v>252</v>
       </c>
       <c r="C657" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D657" t="s">
         <v>323</v>
@@ -71223,7 +71223,7 @@
         <v>46241</v>
       </c>
       <c r="I657" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J657" s="7">
         <v>0.02</v>
@@ -71437,7 +71437,7 @@
         <v>46308</v>
       </c>
       <c r="I659" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J659" s="7">
         <v>0.35</v>
@@ -71972,7 +71972,7 @@
         <v>46426</v>
       </c>
       <c r="I664" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J664" s="7">
         <v>4</v>
@@ -72489,7 +72489,7 @@
         <v>252</v>
       </c>
       <c r="C669" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D669" t="s">
         <v>166</v>
@@ -72507,7 +72507,7 @@
         <v>46752</v>
       </c>
       <c r="I669" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J669" s="7">
         <v>14</v>
@@ -72709,7 +72709,7 @@
         <v>166</v>
       </c>
       <c r="E671" s="12" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="F671" t="s">
         <v>252</v>
@@ -73256,7 +73256,7 @@
         <v>46349</v>
       </c>
       <c r="I676" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J676" t="s">
         <v>252</v>
@@ -73684,7 +73684,7 @@
         <v>47003</v>
       </c>
       <c r="I680" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J680" t="s">
         <v>252</v>
@@ -73898,7 +73898,7 @@
         <v>47003</v>
       </c>
       <c r="I682" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J682" t="s">
         <v>252</v>
@@ -74112,7 +74112,7 @@
         <v>46387</v>
       </c>
       <c r="I684" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J684" t="s">
         <v>252</v>
@@ -74326,7 +74326,7 @@
         <v>46387</v>
       </c>
       <c r="I686" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J686" t="s">
         <v>252</v>
@@ -74540,7 +74540,7 @@
         <v>46387</v>
       </c>
       <c r="I688" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J688" t="s">
         <v>252</v>
@@ -74736,7 +74736,7 @@
         <v>252</v>
       </c>
       <c r="C690" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D690" t="s">
         <v>108</v>
@@ -74754,7 +74754,7 @@
         <v>46387</v>
       </c>
       <c r="I690" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J690" t="s">
         <v>252</v>
@@ -74968,7 +74968,7 @@
         <v>252</v>
       </c>
       <c r="I692" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J692" s="7">
         <v>10.54</v>
@@ -75075,7 +75075,7 @@
         <v>51936</v>
       </c>
       <c r="I693" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J693" s="7">
         <v>0.04</v>
@@ -75717,7 +75717,7 @@
         <v>46387</v>
       </c>
       <c r="I699" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J699" t="s">
         <v>252</v>
@@ -75931,7 +75931,7 @@
         <v>46387</v>
       </c>
       <c r="I701" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J701" t="s">
         <v>252</v>
@@ -76145,7 +76145,7 @@
         <v>45443</v>
       </c>
       <c r="I703" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J703" t="s">
         <v>252</v>
@@ -76359,7 +76359,7 @@
         <v>46022</v>
       </c>
       <c r="I705" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J705" t="s">
         <v>252</v>
@@ -76573,7 +76573,7 @@
         <v>46387</v>
       </c>
       <c r="I707" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J707" s="5" t="s">
         <v>252</v>
@@ -76787,7 +76787,7 @@
         <v>46387</v>
       </c>
       <c r="I709" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J709" t="s">
         <v>252</v>
@@ -77001,7 +77001,7 @@
         <v>46387</v>
       </c>
       <c r="I711" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J711" t="s">
         <v>252</v>
@@ -77215,7 +77215,7 @@
         <v>46349</v>
       </c>
       <c r="I713" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J713" s="7">
         <v>2.5</v>
@@ -77536,7 +77536,7 @@
         <v>47003</v>
       </c>
       <c r="I716" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J716" t="s">
         <v>252</v>
@@ -77750,7 +77750,7 @@
         <v>47003</v>
       </c>
       <c r="I718" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J718" t="s">
         <v>252</v>
@@ -77964,7 +77964,7 @@
         <v>46387</v>
       </c>
       <c r="I720" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J720" t="s">
         <v>252</v>
@@ -78178,7 +78178,7 @@
         <v>46387</v>
       </c>
       <c r="I722" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J722" t="s">
         <v>252</v>
@@ -78392,7 +78392,7 @@
         <v>46387</v>
       </c>
       <c r="I724" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J724" t="s">
         <v>252</v>
@@ -78588,7 +78588,7 @@
         <v>252</v>
       </c>
       <c r="C726" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D726" t="s">
         <v>108</v>
@@ -78606,7 +78606,7 @@
         <v>46387</v>
       </c>
       <c r="I726" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J726" t="s">
         <v>252</v>
@@ -78820,7 +78820,7 @@
         <v>46213</v>
       </c>
       <c r="I728" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J728" s="7">
         <v>8</v>

</xml_diff>

<commit_message>
Update schedule via dashboard 2026-08-11T20:03:03.447Z
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -373,9 +373,6 @@
     <t>Rockdale County, GA</t>
   </si>
   <si>
-    <t>First Name</t>
-  </si>
-  <si>
     <t>Jefferson County Commission</t>
   </si>
   <si>
@@ -467,6 +464,9 @@
   </si>
   <si>
     <t>Pace Water</t>
+  </si>
+  <si>
+    <t>Conversion Documentation &amp; Updates - Take 2</t>
   </si>
   <si>
     <t>Time Off - Stat. Holidays</t>
@@ -622,6 +622,9 @@
     <t>Jean</t>
   </si>
   <si>
+    <t>Roanoke Gas Company</t>
+  </si>
+  <si>
     <t>Go-Live</t>
   </si>
   <si>
@@ -749,9 +752,6 @@
   </si>
   <si>
     <t>Weekly Internal Project Meetings 12</t>
-  </si>
-  <si>
-    <t>Generated on behalf of Ali Raoofi on Tuesday, August 11, 2026 2:55:35 PM</t>
   </si>
   <si>
     <t>Weekly Client Meetings 79</t>
@@ -1012,7 +1012,7 @@
     <t>Disconnect Customization - PS Functional Testing</t>
   </si>
   <si>
-    <t>Conversion Documentation &amp; Updates - Take 2</t>
+    <t>First Name</t>
   </si>
   <si>
     <t>z-Cogsdale - Internal Cloud Maintenance</t>
@@ -1145,7 +1145,7 @@
     <t>Weekly Internal Project Meetings 30</t>
   </si>
   <si>
-    <t>Roanoke Gas Company</t>
+    <t>Generated on behalf of Ali Raoofi on Tuesday, August 11, 2026 3:02:20 PM</t>
   </si>
   <si>
     <t>Integration planning including touch points, business process changes, and business best practices/ impacts/risks</t>
@@ -1969,7 +1969,7 @@
     </row>
     <row r="5" spans="1:34" ht="12.75" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>239</v>
+        <v>368</v>
       </c>
     </row>
     <row r="7" spans="1:34" ht="18.75" customHeight="1">
@@ -1979,13 +1979,13 @@
     </row>
     <row r="9" spans="1:34" ht="25.5" customHeight="1">
       <c r="A9" s="3" t="s">
-        <v>116</v>
+        <v>325</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>375</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>11</v>
@@ -2000,7 +2000,7 @@
         <v>307</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>4</v>
@@ -2039,16 +2039,16 @@
         <v>90</v>
       </c>
       <c r="U9" s="4" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="V9" s="4" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="W9" s="4" t="s">
         <v>163</v>
       </c>
       <c r="X9" s="4" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="Y9" s="4" t="s">
         <v>305</v>
@@ -2060,7 +2060,7 @@
         <v>164</v>
       </c>
       <c r="AB9" s="4" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AC9" s="4" t="s">
         <v>365</v>
@@ -2069,7 +2069,7 @@
         <v>288</v>
       </c>
       <c r="AE9" s="4" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="AF9" s="4" t="s">
         <v>410</v>
@@ -2078,7 +2078,7 @@
         <v>169</v>
       </c>
       <c r="AH9" s="4" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="10" spans="1:34" ht="12.75" customHeight="1">
@@ -2107,61 +2107,61 @@
         <v>267</v>
       </c>
       <c r="I10" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J10" s="6">
-        <v>241.29</v>
+        <v>221.29</v>
       </c>
       <c r="K10" s="6">
-        <v>221.59</v>
+        <v>241.59</v>
       </c>
       <c r="L10" s="6">
         <v>164.33</v>
       </c>
       <c r="M10" s="6">
-        <v>186.93</v>
+        <v>183.93</v>
       </c>
       <c r="N10" s="6">
-        <v>188.54</v>
-      </c>
-      <c r="O10" s="6">
-        <v>220.07</v>
+        <v>185.54</v>
+      </c>
+      <c r="O10" s="7">
+        <v>102.73</v>
       </c>
       <c r="P10" s="6">
-        <v>190.86</v>
+        <v>190.99</v>
       </c>
       <c r="Q10" s="6">
-        <v>152.32</v>
+        <v>152.45</v>
       </c>
       <c r="R10" s="7">
-        <v>131.94</v>
+        <v>132.08</v>
       </c>
       <c r="S10" s="6">
-        <v>160.02</v>
+        <v>160.15</v>
       </c>
       <c r="T10" s="6">
-        <v>171.32</v>
+        <v>171.45</v>
       </c>
       <c r="U10" s="6">
-        <v>144.9</v>
+        <v>145.04</v>
       </c>
       <c r="V10" s="6">
-        <v>134.24</v>
+        <v>254.37</v>
       </c>
       <c r="W10" s="6">
-        <v>195.74</v>
+        <v>195.87</v>
       </c>
       <c r="X10" s="6">
-        <v>167.24</v>
+        <v>167.37</v>
       </c>
       <c r="Y10" s="6">
-        <v>244.24</v>
+        <v>244.37</v>
       </c>
       <c r="Z10" s="6">
-        <v>192.02</v>
+        <v>192.16</v>
       </c>
       <c r="AA10" s="6">
-        <v>156.56</v>
+        <v>156.7</v>
       </c>
       <c r="AB10" s="6">
         <v>153.83</v>
@@ -2211,7 +2211,7 @@
         <v>267</v>
       </c>
       <c r="I11" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J11" s="7">
         <v>34.5</v>
@@ -2315,7 +2315,7 @@
         <v>51936</v>
       </c>
       <c r="I12" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J12" s="7">
         <v>27.5</v>
@@ -2407,7 +2407,7 @@
         <v>417</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F13" t="s">
         <v>267</v>
@@ -2921,7 +2921,7 @@
         <v>267</v>
       </c>
       <c r="C18" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D18" t="s">
         <v>392</v>
@@ -2930,7 +2930,7 @@
         <v>392</v>
       </c>
       <c r="F18" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="G18" s="10">
         <v>45569</v>
@@ -2939,7 +2939,7 @@
         <v>46262</v>
       </c>
       <c r="I18" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J18" s="7">
         <v>2</v>
@@ -3129,7 +3129,7 @@
         <v>267</v>
       </c>
       <c r="C20" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D20" t="s">
         <v>173</v>
@@ -3147,7 +3147,7 @@
         <v>47079</v>
       </c>
       <c r="I20" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J20" s="7">
         <v>1</v>
@@ -3441,7 +3441,7 @@
         <v>267</v>
       </c>
       <c r="C23" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D23" t="s">
         <v>111</v>
@@ -3450,7 +3450,7 @@
         <v>111</v>
       </c>
       <c r="F23" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="G23" s="10">
         <v>46101</v>
@@ -3459,7 +3459,7 @@
         <v>46262</v>
       </c>
       <c r="I23" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J23" s="7">
         <v>3</v>
@@ -3649,7 +3649,7 @@
         <v>267</v>
       </c>
       <c r="C25" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D25" t="s">
         <v>256</v>
@@ -3667,7 +3667,7 @@
         <v>46304</v>
       </c>
       <c r="I25" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J25" t="s">
         <v>267</v>
@@ -3857,7 +3857,7 @@
         <v>267</v>
       </c>
       <c r="C27" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D27" t="s">
         <v>389</v>
@@ -3875,7 +3875,7 @@
         <v>46387</v>
       </c>
       <c r="I27" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J27" s="7">
         <v>1</v>
@@ -4175,7 +4175,7 @@
         <v>389</v>
       </c>
       <c r="E30" s="11" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="F30" t="s">
         <v>267</v>
@@ -4707,7 +4707,7 @@
         <v>267</v>
       </c>
       <c r="I35" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J35" s="7">
         <v>33.33</v>
@@ -4811,7 +4811,7 @@
         <v>51936</v>
       </c>
       <c r="I36" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J36" s="7">
         <v>32.5</v>
@@ -4903,7 +4903,7 @@
         <v>417</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F37" t="s">
         <v>267</v>
@@ -5423,7 +5423,7 @@
         <v>417</v>
       </c>
       <c r="E42" s="11" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F42" t="s">
         <v>267</v>
@@ -5539,7 +5539,7 @@
         <v>46267</v>
       </c>
       <c r="I43" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J43" s="7">
         <v>0.83</v>
@@ -5631,7 +5631,7 @@
         <v>1</v>
       </c>
       <c r="E44" s="11" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F44" t="s">
         <v>267</v>
@@ -5830,7 +5830,7 @@
         <v>52</v>
       </c>
       <c r="B46" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C46" t="s">
         <v>267</v>
@@ -5851,13 +5851,13 @@
         <v>267</v>
       </c>
       <c r="I46" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J46" s="7">
-        <v>37.33</v>
+        <v>17.33</v>
       </c>
       <c r="K46" s="12">
-        <v>40.73</v>
+        <v>60.73</v>
       </c>
       <c r="L46" s="7">
         <v>20.1</v>
@@ -5868,8 +5868,8 @@
       <c r="N46" s="7">
         <v>18</v>
       </c>
-      <c r="O46" s="12">
-        <v>49.5</v>
+      <c r="O46" s="7">
+        <v>9.5</v>
       </c>
       <c r="P46" s="6">
         <v>38.5</v>
@@ -5889,8 +5889,8 @@
       <c r="U46" s="7">
         <v>30.38</v>
       </c>
-      <c r="V46" s="7">
-        <v>18.38</v>
+      <c r="V46" s="12">
+        <v>58.38</v>
       </c>
       <c r="W46" s="12">
         <v>57.38</v>
@@ -5955,7 +5955,7 @@
         <v>51936</v>
       </c>
       <c r="I47" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J47" s="7">
         <v>12.5</v>
@@ -6047,7 +6047,7 @@
         <v>417</v>
       </c>
       <c r="E48" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F48" t="s">
         <v>267</v>
@@ -6579,7 +6579,7 @@
         <v>46325</v>
       </c>
       <c r="I53" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J53" t="s">
         <v>267</v>
@@ -6671,7 +6671,7 @@
         <v>355</v>
       </c>
       <c r="E54" s="11" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F54" t="s">
         <v>267</v>
@@ -6778,7 +6778,7 @@
         <v>346</v>
       </c>
       <c r="F55" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="G55" s="10">
         <v>44837</v>
@@ -6787,7 +6787,7 @@
         <v>46387</v>
       </c>
       <c r="I55" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J55" t="s">
         <v>267</v>
@@ -6995,7 +6995,7 @@
         <v>46267</v>
       </c>
       <c r="I57" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J57" s="7">
         <v>0.83</v>
@@ -7087,7 +7087,7 @@
         <v>1</v>
       </c>
       <c r="E58" s="11" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F58" t="s">
         <v>267</v>
@@ -7289,7 +7289,7 @@
         <v>267</v>
       </c>
       <c r="C60" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D60" t="s">
         <v>171</v>
@@ -7307,7 +7307,7 @@
         <v>46493</v>
       </c>
       <c r="I60" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J60" s="7">
         <v>3</v>
@@ -8127,7 +8127,7 @@
         <v>171</v>
       </c>
       <c r="E68" s="11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F68" t="s">
         <v>267</v>
@@ -8231,7 +8231,7 @@
         <v>171</v>
       </c>
       <c r="E69" s="11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F69" t="s">
         <v>267</v>
@@ -12195,7 +12195,7 @@
         <v>46416</v>
       </c>
       <c r="I107" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J107" t="s">
         <v>267</v>
@@ -12212,8 +12212,8 @@
       <c r="N107" t="s">
         <v>267</v>
       </c>
-      <c r="O107" s="12">
-        <v>40</v>
+      <c r="O107" t="s">
+        <v>267</v>
       </c>
       <c r="P107" t="s">
         <v>267</v>
@@ -12233,8 +12233,8 @@
       <c r="U107" s="7">
         <v>0.5</v>
       </c>
-      <c r="V107" s="7">
-        <v>0.5</v>
+      <c r="V107" s="12">
+        <v>40.5</v>
       </c>
       <c r="W107" s="7">
         <v>0.5</v>
@@ -12495,7 +12495,7 @@
         <v>46</v>
       </c>
       <c r="E110" s="11" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F110" t="s">
         <v>267</v>
@@ -12599,16 +12599,16 @@
         <v>46</v>
       </c>
       <c r="E111" s="11" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="F111" t="s">
         <v>267</v>
       </c>
       <c r="G111" s="10">
-        <v>46279</v>
+        <v>46293</v>
       </c>
       <c r="H111" s="10">
-        <v>46283</v>
+        <v>46304</v>
       </c>
       <c r="I111" t="s">
         <v>267</v>
@@ -12628,17 +12628,17 @@
       <c r="N111" t="s">
         <v>267</v>
       </c>
-      <c r="O111" s="12">
-        <v>40</v>
+      <c r="O111" t="s">
+        <v>267</v>
       </c>
       <c r="P111" t="s">
         <v>267</v>
       </c>
-      <c r="Q111" t="s">
-        <v>267</v>
-      </c>
-      <c r="R111" t="s">
-        <v>267</v>
+      <c r="Q111" s="7">
+        <v>2.5</v>
+      </c>
+      <c r="R111" s="7">
+        <v>2.5</v>
       </c>
       <c r="S111" t="s">
         <v>267</v>
@@ -12703,16 +12703,16 @@
         <v>46</v>
       </c>
       <c r="E112" s="11" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="F112" t="s">
         <v>267</v>
       </c>
       <c r="G112" s="10">
-        <v>46293</v>
+        <v>46328</v>
       </c>
       <c r="H112" s="10">
-        <v>46304</v>
+        <v>46332</v>
       </c>
       <c r="I112" t="s">
         <v>267</v>
@@ -12738,11 +12738,11 @@
       <c r="P112" t="s">
         <v>267</v>
       </c>
-      <c r="Q112" s="7">
-        <v>2.5</v>
-      </c>
-      <c r="R112" s="7">
-        <v>2.5</v>
+      <c r="Q112" t="s">
+        <v>267</v>
+      </c>
+      <c r="R112" t="s">
+        <v>267</v>
       </c>
       <c r="S112" t="s">
         <v>267</v>
@@ -12753,8 +12753,8 @@
       <c r="U112" t="s">
         <v>267</v>
       </c>
-      <c r="V112" t="s">
-        <v>267</v>
+      <c r="V112" s="12">
+        <v>40</v>
       </c>
       <c r="W112" t="s">
         <v>267</v>
@@ -13431,7 +13431,7 @@
         <v>46</v>
       </c>
       <c r="E119" s="11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F119" t="s">
         <v>267</v>
@@ -13529,7 +13529,7 @@
         <v>267</v>
       </c>
       <c r="C120" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D120" t="s">
         <v>173</v>
@@ -13547,13 +13547,13 @@
         <v>47079</v>
       </c>
       <c r="I120" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J120" s="7">
-        <v>21</v>
-      </c>
-      <c r="K120" t="s">
-        <v>267</v>
+        <v>1</v>
+      </c>
+      <c r="K120" s="7">
+        <v>20</v>
       </c>
       <c r="L120" s="7">
         <v>1</v>
@@ -13752,16 +13752,16 @@
         <v>46227</v>
       </c>
       <c r="H122" s="10">
-        <v>46248</v>
+        <v>46255</v>
       </c>
       <c r="I122" t="s">
         <v>267</v>
       </c>
-      <c r="J122" s="7">
+      <c r="J122" t="s">
+        <v>267</v>
+      </c>
+      <c r="K122" s="7">
         <v>20</v>
-      </c>
-      <c r="K122" t="s">
-        <v>267</v>
       </c>
       <c r="L122" t="s">
         <v>267</v>
@@ -15095,7 +15095,7 @@
         <v>173</v>
       </c>
       <c r="E135" s="11" t="s">
-        <v>325</v>
+        <v>147</v>
       </c>
       <c r="F135" t="s">
         <v>267</v>
@@ -15315,7 +15315,7 @@
         <v>46454</v>
       </c>
       <c r="I137" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J137" t="s">
         <v>267</v>
@@ -15921,7 +15921,7 @@
         <v>267</v>
       </c>
       <c r="C143" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D143" t="s">
         <v>156</v>
@@ -15939,7 +15939,7 @@
         <v>46531</v>
       </c>
       <c r="I143" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J143" t="s">
         <v>267</v>
@@ -16441,7 +16441,7 @@
         <v>267</v>
       </c>
       <c r="C148" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D148" t="s">
         <v>111</v>
@@ -16450,7 +16450,7 @@
         <v>111</v>
       </c>
       <c r="F148" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="G148" s="10">
         <v>46101</v>
@@ -16459,7 +16459,7 @@
         <v>46262</v>
       </c>
       <c r="I148" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J148" t="s">
         <v>267</v>
@@ -16649,7 +16649,7 @@
         <v>267</v>
       </c>
       <c r="C150" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D150" t="s">
         <v>24</v>
@@ -16658,7 +16658,7 @@
         <v>24</v>
       </c>
       <c r="F150" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G150" s="10">
         <v>46114</v>
@@ -16667,7 +16667,7 @@
         <v>46283</v>
       </c>
       <c r="I150" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J150" t="s">
         <v>267</v>
@@ -16759,7 +16759,7 @@
         <v>24</v>
       </c>
       <c r="E151" s="11" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F151" t="s">
         <v>267</v>
@@ -16857,7 +16857,7 @@
         <v>267</v>
       </c>
       <c r="C152" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D152" t="s">
         <v>256</v>
@@ -16875,7 +16875,7 @@
         <v>46304</v>
       </c>
       <c r="I152" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J152" t="s">
         <v>267</v>
@@ -17083,7 +17083,7 @@
         <v>46248</v>
       </c>
       <c r="I154" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J154" t="s">
         <v>267</v>
@@ -17291,7 +17291,7 @@
         <v>46356</v>
       </c>
       <c r="I156" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J156" t="s">
         <v>267</v>
@@ -17383,7 +17383,7 @@
         <v>160</v>
       </c>
       <c r="E157" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F157" t="s">
         <v>267</v>
@@ -17585,7 +17585,7 @@
         <v>267</v>
       </c>
       <c r="C159" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D159" t="s">
         <v>389</v>
@@ -17603,7 +17603,7 @@
         <v>46387</v>
       </c>
       <c r="I159" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J159" t="s">
         <v>267</v>
@@ -17811,7 +17811,7 @@
         <v>46498</v>
       </c>
       <c r="I161" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J161" t="s">
         <v>267</v>
@@ -17903,7 +17903,7 @@
         <v>63</v>
       </c>
       <c r="E162" s="11" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F162" t="s">
         <v>267</v>
@@ -18539,7 +18539,7 @@
         <v>267</v>
       </c>
       <c r="I168" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J168" t="s">
         <v>267</v>
@@ -18643,7 +18643,7 @@
         <v>51936</v>
       </c>
       <c r="I169" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J169" t="s">
         <v>267</v>
@@ -18851,7 +18851,7 @@
         <v>46315</v>
       </c>
       <c r="I171" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J171" t="s">
         <v>267</v>
@@ -18943,7 +18943,7 @@
         <v>87</v>
       </c>
       <c r="E172" s="11" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F172" t="s">
         <v>267</v>
@@ -19163,7 +19163,7 @@
         <v>267</v>
       </c>
       <c r="I174" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J174" s="7">
         <v>21.5</v>
@@ -19180,8 +19180,8 @@
       <c r="N174" s="7">
         <v>24.24</v>
       </c>
-      <c r="O174" s="12">
-        <v>58.24</v>
+      <c r="O174" s="7">
+        <v>18.24</v>
       </c>
       <c r="P174" s="12">
         <v>47.8</v>
@@ -19201,8 +19201,8 @@
       <c r="U174" s="7">
         <v>9.07</v>
       </c>
-      <c r="V174" s="7">
-        <v>8.73</v>
+      <c r="V174" s="12">
+        <v>48.73</v>
       </c>
       <c r="W174" s="7">
         <v>8.73</v>
@@ -19267,7 +19267,7 @@
         <v>51936</v>
       </c>
       <c r="I175" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J175" s="7">
         <v>7.5</v>
@@ -19359,7 +19359,7 @@
         <v>417</v>
       </c>
       <c r="E176" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F176" t="s">
         <v>267</v>
@@ -19891,7 +19891,7 @@
         <v>46325</v>
       </c>
       <c r="I181" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J181" s="7">
         <v>5</v>
@@ -19983,7 +19983,7 @@
         <v>355</v>
       </c>
       <c r="E182" s="11" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F182" t="s">
         <v>267</v>
@@ -20099,7 +20099,7 @@
         <v>46259</v>
       </c>
       <c r="I183" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J183" s="7">
         <v>7.5</v>
@@ -20307,7 +20307,7 @@
         <v>46267</v>
       </c>
       <c r="I185" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J185" t="s">
         <v>267</v>
@@ -20515,7 +20515,7 @@
         <v>46416</v>
       </c>
       <c r="I187" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J187" s="7">
         <v>1</v>
@@ -20532,8 +20532,8 @@
       <c r="N187" s="7">
         <v>1</v>
       </c>
-      <c r="O187" s="12">
-        <v>43</v>
+      <c r="O187" s="7">
+        <v>3</v>
       </c>
       <c r="P187" s="7">
         <v>3</v>
@@ -20553,8 +20553,8 @@
       <c r="U187" s="7">
         <v>1</v>
       </c>
-      <c r="V187" s="7">
-        <v>1</v>
+      <c r="V187" s="12">
+        <v>41</v>
       </c>
       <c r="W187" s="7">
         <v>1</v>
@@ -20815,7 +20815,7 @@
         <v>46</v>
       </c>
       <c r="E190" s="11" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F190" t="s">
         <v>267</v>
@@ -21023,16 +21023,16 @@
         <v>46</v>
       </c>
       <c r="E192" s="11" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="F192" t="s">
         <v>267</v>
       </c>
       <c r="G192" s="10">
-        <v>46279</v>
+        <v>46293</v>
       </c>
       <c r="H192" s="10">
-        <v>46283</v>
+        <v>46304</v>
       </c>
       <c r="I192" t="s">
         <v>267</v>
@@ -21052,17 +21052,17 @@
       <c r="N192" t="s">
         <v>267</v>
       </c>
-      <c r="O192" s="12">
-        <v>40</v>
+      <c r="O192" t="s">
+        <v>267</v>
       </c>
       <c r="P192" t="s">
         <v>267</v>
       </c>
-      <c r="Q192" t="s">
-        <v>267</v>
-      </c>
-      <c r="R192" t="s">
-        <v>267</v>
+      <c r="Q192" s="7">
+        <v>2.5</v>
+      </c>
+      <c r="R192" s="7">
+        <v>2.5</v>
       </c>
       <c r="S192" t="s">
         <v>267</v>
@@ -21127,16 +21127,16 @@
         <v>46</v>
       </c>
       <c r="E193" s="11" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="F193" t="s">
         <v>267</v>
       </c>
       <c r="G193" s="10">
-        <v>46293</v>
+        <v>46328</v>
       </c>
       <c r="H193" s="10">
-        <v>46304</v>
+        <v>46332</v>
       </c>
       <c r="I193" t="s">
         <v>267</v>
@@ -21162,11 +21162,11 @@
       <c r="P193" t="s">
         <v>267</v>
       </c>
-      <c r="Q193" s="7">
-        <v>2.5</v>
-      </c>
-      <c r="R193" s="7">
-        <v>2.5</v>
+      <c r="Q193" t="s">
+        <v>267</v>
+      </c>
+      <c r="R193" t="s">
+        <v>267</v>
       </c>
       <c r="S193" t="s">
         <v>267</v>
@@ -21177,8 +21177,8 @@
       <c r="U193" t="s">
         <v>267</v>
       </c>
-      <c r="V193" t="s">
-        <v>267</v>
+      <c r="V193" s="12">
+        <v>40</v>
       </c>
       <c r="W193" t="s">
         <v>267</v>
@@ -21855,7 +21855,7 @@
         <v>46</v>
       </c>
       <c r="E200" s="11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F200" t="s">
         <v>267</v>
@@ -21971,7 +21971,7 @@
         <v>46454</v>
       </c>
       <c r="I201" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J201" t="s">
         <v>267</v>
@@ -22161,7 +22161,7 @@
         <v>267</v>
       </c>
       <c r="C203" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D203" t="s">
         <v>156</v>
@@ -22179,7 +22179,7 @@
         <v>46531</v>
       </c>
       <c r="I203" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J203" t="s">
         <v>267</v>
@@ -22577,7 +22577,7 @@
         <v>267</v>
       </c>
       <c r="C207" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D207" t="s">
         <v>256</v>
@@ -22595,7 +22595,7 @@
         <v>46304</v>
       </c>
       <c r="I207" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J207" t="s">
         <v>267</v>
@@ -22803,7 +22803,7 @@
         <v>46356</v>
       </c>
       <c r="I209" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J209" t="s">
         <v>267</v>
@@ -23103,7 +23103,7 @@
         <v>160</v>
       </c>
       <c r="E212" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F212" t="s">
         <v>267</v>
@@ -23513,7 +23513,7 @@
         <v>267</v>
       </c>
       <c r="C216" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D216" t="s">
         <v>389</v>
@@ -23531,7 +23531,7 @@
         <v>46387</v>
       </c>
       <c r="I216" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J216" s="7">
         <v>0.5</v>
@@ -23831,7 +23831,7 @@
         <v>389</v>
       </c>
       <c r="E219" s="11" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="F219" t="s">
         <v>267</v>
@@ -24345,7 +24345,7 @@
         <v>267</v>
       </c>
       <c r="C224" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D224" t="s">
         <v>103</v>
@@ -24363,7 +24363,7 @@
         <v>46325</v>
       </c>
       <c r="I224" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J224" t="s">
         <v>267</v>
@@ -24767,7 +24767,7 @@
         <v>103</v>
       </c>
       <c r="E228" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F228" t="s">
         <v>267</v>
@@ -24871,7 +24871,7 @@
         <v>267</v>
       </c>
       <c r="E229" s="8" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F229" t="s">
         <v>267</v>
@@ -24883,7 +24883,7 @@
         <v>267</v>
       </c>
       <c r="I229" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J229" s="7">
         <v>16.83</v>
@@ -24987,7 +24987,7 @@
         <v>51936</v>
       </c>
       <c r="I230" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J230" s="7">
         <v>7.5</v>
@@ -25079,7 +25079,7 @@
         <v>417</v>
       </c>
       <c r="E231" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F231" t="s">
         <v>267</v>
@@ -25611,7 +25611,7 @@
         <v>46259</v>
       </c>
       <c r="I236" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J236" s="7">
         <v>7.5</v>
@@ -25819,7 +25819,7 @@
         <v>46267</v>
       </c>
       <c r="I238" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J238" s="7">
         <v>0.83</v>
@@ -25911,7 +25911,7 @@
         <v>1</v>
       </c>
       <c r="E239" s="11" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F239" t="s">
         <v>267</v>
@@ -26113,7 +26113,7 @@
         <v>267</v>
       </c>
       <c r="C241" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D241" t="s">
         <v>173</v>
@@ -26131,7 +26131,7 @@
         <v>47079</v>
       </c>
       <c r="I241" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J241" t="s">
         <v>267</v>
@@ -26951,7 +26951,7 @@
         <v>173</v>
       </c>
       <c r="E249" s="11" t="s">
-        <v>325</v>
+        <v>147</v>
       </c>
       <c r="F249" t="s">
         <v>267</v>
@@ -27171,7 +27171,7 @@
         <v>46248</v>
       </c>
       <c r="I251" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J251" s="7">
         <v>1</v>
@@ -27379,7 +27379,7 @@
         <v>267</v>
       </c>
       <c r="I253" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J253" s="12">
         <v>39.5</v>
@@ -27391,49 +27391,49 @@
         <v>22.5</v>
       </c>
       <c r="M253" s="12">
-        <v>52.5</v>
+        <v>49.5</v>
       </c>
       <c r="N253" s="12">
-        <v>60</v>
-      </c>
-      <c r="O253" s="12">
-        <v>52.5</v>
+        <v>57</v>
+      </c>
+      <c r="O253" s="7">
+        <v>15.17</v>
       </c>
       <c r="P253" s="6">
-        <v>28.07</v>
+        <v>28.2</v>
       </c>
       <c r="Q253" s="7">
-        <v>24.57</v>
+        <v>24.7</v>
       </c>
       <c r="R253" s="7">
-        <v>24.57</v>
+        <v>24.7</v>
       </c>
       <c r="S253" s="12">
-        <v>49.77</v>
+        <v>49.9</v>
       </c>
       <c r="T253" s="12">
-        <v>70.57</v>
+        <v>70.7</v>
       </c>
       <c r="U253" s="12">
-        <v>47.9</v>
+        <v>48.03</v>
       </c>
       <c r="V253" s="12">
-        <v>41.9</v>
+        <v>82.03</v>
       </c>
       <c r="W253" s="12">
-        <v>41.9</v>
+        <v>42.03</v>
       </c>
       <c r="X253" s="12">
-        <v>41.9</v>
+        <v>42.03</v>
       </c>
       <c r="Y253" s="12">
-        <v>71.9</v>
+        <v>72.03</v>
       </c>
       <c r="Z253" s="6">
-        <v>37.9</v>
+        <v>38.03</v>
       </c>
       <c r="AA253" s="7">
-        <v>18.57</v>
+        <v>18.7</v>
       </c>
       <c r="AB253" s="7">
         <v>24.8</v>
@@ -27483,7 +27483,7 @@
         <v>51936</v>
       </c>
       <c r="I254" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J254" s="7">
         <v>7.5</v>
@@ -27575,7 +27575,7 @@
         <v>417</v>
       </c>
       <c r="E255" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F255" t="s">
         <v>267</v>
@@ -28098,7 +28098,7 @@
         <v>346</v>
       </c>
       <c r="F260" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="G260" s="10">
         <v>44837</v>
@@ -28107,7 +28107,7 @@
         <v>46387</v>
       </c>
       <c r="I260" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J260" t="s">
         <v>267</v>
@@ -28315,7 +28315,7 @@
         <v>46259</v>
       </c>
       <c r="I262" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J262" s="7">
         <v>11.5</v>
@@ -28609,7 +28609,7 @@
         <v>267</v>
       </c>
       <c r="C265" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D265" t="s">
         <v>171</v>
@@ -28627,7 +28627,7 @@
         <v>46493</v>
       </c>
       <c r="I265" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J265" s="7">
         <v>16.5</v>
@@ -29447,7 +29447,7 @@
         <v>171</v>
       </c>
       <c r="E273" s="11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F273" t="s">
         <v>267</v>
@@ -29551,7 +29551,7 @@
         <v>171</v>
       </c>
       <c r="E274" s="11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F274" t="s">
         <v>267</v>
@@ -33307,7 +33307,7 @@
         <v>46416</v>
       </c>
       <c r="I310" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J310" t="s">
         <v>267</v>
@@ -33324,29 +33324,29 @@
       <c r="N310" t="s">
         <v>267</v>
       </c>
-      <c r="O310" s="12">
+      <c r="O310" t="s">
+        <v>267</v>
+      </c>
+      <c r="P310" t="s">
+        <v>267</v>
+      </c>
+      <c r="Q310" t="s">
+        <v>267</v>
+      </c>
+      <c r="R310" t="s">
+        <v>267</v>
+      </c>
+      <c r="S310" t="s">
+        <v>267</v>
+      </c>
+      <c r="T310" t="s">
+        <v>267</v>
+      </c>
+      <c r="U310" t="s">
+        <v>267</v>
+      </c>
+      <c r="V310" s="12">
         <v>40</v>
-      </c>
-      <c r="P310" t="s">
-        <v>267</v>
-      </c>
-      <c r="Q310" t="s">
-        <v>267</v>
-      </c>
-      <c r="R310" t="s">
-        <v>267</v>
-      </c>
-      <c r="S310" t="s">
-        <v>267</v>
-      </c>
-      <c r="T310" t="s">
-        <v>267</v>
-      </c>
-      <c r="U310" t="s">
-        <v>267</v>
-      </c>
-      <c r="V310" t="s">
-        <v>267</v>
       </c>
       <c r="W310" t="s">
         <v>267</v>
@@ -33399,16 +33399,16 @@
         <v>46</v>
       </c>
       <c r="E311" s="11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F311" t="s">
         <v>267</v>
       </c>
       <c r="G311" s="10">
-        <v>46279</v>
+        <v>46328</v>
       </c>
       <c r="H311" s="10">
-        <v>46283</v>
+        <v>46332</v>
       </c>
       <c r="I311" t="s">
         <v>267</v>
@@ -33428,29 +33428,29 @@
       <c r="N311" t="s">
         <v>267</v>
       </c>
-      <c r="O311" s="12">
+      <c r="O311" t="s">
+        <v>267</v>
+      </c>
+      <c r="P311" t="s">
+        <v>267</v>
+      </c>
+      <c r="Q311" t="s">
+        <v>267</v>
+      </c>
+      <c r="R311" t="s">
+        <v>267</v>
+      </c>
+      <c r="S311" t="s">
+        <v>267</v>
+      </c>
+      <c r="T311" t="s">
+        <v>267</v>
+      </c>
+      <c r="U311" t="s">
+        <v>267</v>
+      </c>
+      <c r="V311" s="12">
         <v>40</v>
-      </c>
-      <c r="P311" t="s">
-        <v>267</v>
-      </c>
-      <c r="Q311" t="s">
-        <v>267</v>
-      </c>
-      <c r="R311" t="s">
-        <v>267</v>
-      </c>
-      <c r="S311" t="s">
-        <v>267</v>
-      </c>
-      <c r="T311" t="s">
-        <v>267</v>
-      </c>
-      <c r="U311" t="s">
-        <v>267</v>
-      </c>
-      <c r="V311" t="s">
-        <v>267</v>
       </c>
       <c r="W311" t="s">
         <v>267</v>
@@ -33497,7 +33497,7 @@
         <v>267</v>
       </c>
       <c r="C312" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D312" t="s">
         <v>173</v>
@@ -33515,7 +33515,7 @@
         <v>47079</v>
       </c>
       <c r="I312" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J312" s="7">
         <v>1</v>
@@ -33711,7 +33711,7 @@
         <v>173</v>
       </c>
       <c r="E314" s="11" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F314" t="s">
         <v>267</v>
@@ -34451,7 +34451,7 @@
         <v>46454</v>
       </c>
       <c r="I321" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J321" s="7">
         <v>3</v>
@@ -34462,50 +34462,50 @@
       <c r="L321" s="7">
         <v>3</v>
       </c>
-      <c r="M321" s="7">
-        <v>3</v>
-      </c>
-      <c r="N321" s="7">
-        <v>3</v>
+      <c r="M321" t="s">
+        <v>267</v>
+      </c>
+      <c r="N321" t="s">
+        <v>267</v>
       </c>
       <c r="O321" s="7">
-        <v>3</v>
+        <v>5.67</v>
       </c>
       <c r="P321" s="7">
-        <v>18.57</v>
+        <v>18.7</v>
       </c>
       <c r="Q321" s="7">
-        <v>15.77</v>
+        <v>15.9</v>
       </c>
       <c r="R321" s="7">
-        <v>15.77</v>
+        <v>15.9</v>
       </c>
       <c r="S321" s="7">
-        <v>10.97</v>
+        <v>11.1</v>
       </c>
       <c r="T321" s="7">
-        <v>15.1</v>
+        <v>15.23</v>
       </c>
       <c r="U321" s="7">
-        <v>16.43</v>
+        <v>16.57</v>
       </c>
       <c r="V321" s="7">
-        <v>16.43</v>
+        <v>16.57</v>
       </c>
       <c r="W321" s="7">
-        <v>16.43</v>
+        <v>16.57</v>
       </c>
       <c r="X321" s="7">
-        <v>16.43</v>
+        <v>16.57</v>
       </c>
       <c r="Y321" s="7">
-        <v>16.43</v>
+        <v>16.57</v>
       </c>
       <c r="Z321" s="7">
-        <v>11.1</v>
+        <v>11.23</v>
       </c>
       <c r="AA321" s="7">
-        <v>9.77</v>
+        <v>9.9</v>
       </c>
       <c r="AB321" s="7">
         <v>16</v>
@@ -34566,50 +34566,50 @@
       <c r="L322" s="7">
         <v>1</v>
       </c>
-      <c r="M322" s="7">
-        <v>1</v>
-      </c>
-      <c r="N322" s="7">
-        <v>1</v>
+      <c r="M322" t="s">
+        <v>267</v>
+      </c>
+      <c r="N322" t="s">
+        <v>267</v>
       </c>
       <c r="O322" s="7">
         <v>1</v>
       </c>
       <c r="P322" s="7">
-        <v>9.77</v>
+        <v>9.9</v>
       </c>
       <c r="Q322" s="7">
-        <v>9.77</v>
+        <v>9.9</v>
       </c>
       <c r="R322" s="7">
-        <v>9.77</v>
+        <v>9.9</v>
       </c>
       <c r="S322" s="7">
-        <v>9.77</v>
+        <v>9.9</v>
       </c>
       <c r="T322" s="7">
-        <v>9.77</v>
+        <v>9.9</v>
       </c>
       <c r="U322" s="7">
-        <v>9.77</v>
+        <v>9.9</v>
       </c>
       <c r="V322" s="7">
-        <v>9.77</v>
+        <v>9.9</v>
       </c>
       <c r="W322" s="7">
-        <v>9.77</v>
+        <v>9.9</v>
       </c>
       <c r="X322" s="7">
-        <v>9.77</v>
+        <v>9.9</v>
       </c>
       <c r="Y322" s="7">
-        <v>9.77</v>
+        <v>9.9</v>
       </c>
       <c r="Z322" s="7">
-        <v>9.77</v>
+        <v>9.9</v>
       </c>
       <c r="AA322" s="7">
-        <v>9.77</v>
+        <v>9.9</v>
       </c>
       <c r="AB322" t="s">
         <v>267</v>
@@ -34670,14 +34670,14 @@
       <c r="L323" s="7">
         <v>2</v>
       </c>
-      <c r="M323" s="7">
-        <v>2</v>
-      </c>
-      <c r="N323" s="7">
-        <v>2</v>
+      <c r="M323" t="s">
+        <v>267</v>
+      </c>
+      <c r="N323" t="s">
+        <v>267</v>
       </c>
       <c r="O323" s="7">
-        <v>2</v>
+        <v>4.67</v>
       </c>
       <c r="P323" t="s">
         <v>267</v>
@@ -35473,7 +35473,7 @@
         <v>267</v>
       </c>
       <c r="C331" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D331" t="s">
         <v>24</v>
@@ -35482,7 +35482,7 @@
         <v>24</v>
       </c>
       <c r="F331" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G331" s="10">
         <v>46114</v>
@@ -35491,7 +35491,7 @@
         <v>46283</v>
       </c>
       <c r="I331" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J331" t="s">
         <v>267</v>
@@ -35583,7 +35583,7 @@
         <v>24</v>
       </c>
       <c r="E332" s="11" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F332" t="s">
         <v>267</v>
@@ -35803,7 +35803,7 @@
         <v>267</v>
       </c>
       <c r="I334" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J334" s="12">
         <v>43.6</v>
@@ -35907,7 +35907,7 @@
         <v>51936</v>
       </c>
       <c r="I335" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J335" s="7">
         <v>7.5</v>
@@ -35999,7 +35999,7 @@
         <v>417</v>
       </c>
       <c r="E336" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F336" t="s">
         <v>267</v>
@@ -36513,7 +36513,7 @@
         <v>267</v>
       </c>
       <c r="C341" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D341" t="s">
         <v>173</v>
@@ -36531,7 +36531,7 @@
         <v>47079</v>
       </c>
       <c r="I341" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J341" s="7">
         <v>24</v>
@@ -36831,7 +36831,7 @@
         <v>173</v>
       </c>
       <c r="E344" s="11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F344" t="s">
         <v>267</v>
@@ -37351,7 +37351,7 @@
         <v>173</v>
       </c>
       <c r="E349" s="11" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F349" t="s">
         <v>267</v>
@@ -38079,7 +38079,7 @@
         <v>173</v>
       </c>
       <c r="E356" s="11" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F356" t="s">
         <v>267</v>
@@ -39743,7 +39743,7 @@
         <v>173</v>
       </c>
       <c r="E372" s="11" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F372" t="s">
         <v>267</v>
@@ -39963,7 +39963,7 @@
         <v>46454</v>
       </c>
       <c r="I374" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J374" s="7">
         <v>12.1</v>
@@ -40159,7 +40159,7 @@
         <v>176</v>
       </c>
       <c r="E376" s="11" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F376" t="s">
         <v>267</v>
@@ -40379,7 +40379,7 @@
         <v>267</v>
       </c>
       <c r="I378" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J378" s="7">
         <v>14.69</v>
@@ -40483,7 +40483,7 @@
         <v>51936</v>
       </c>
       <c r="I379" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J379" s="7">
         <v>12.5</v>
@@ -40575,7 +40575,7 @@
         <v>417</v>
       </c>
       <c r="E380" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F380" t="s">
         <v>267</v>
@@ -41089,7 +41089,7 @@
         <v>267</v>
       </c>
       <c r="C385" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D385" t="s">
         <v>173</v>
@@ -41107,7 +41107,7 @@
         <v>47079</v>
       </c>
       <c r="I385" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J385" s="7">
         <v>2.19</v>
@@ -41199,7 +41199,7 @@
         <v>173</v>
       </c>
       <c r="E386" s="11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F386" t="s">
         <v>267</v>
@@ -41823,7 +41823,7 @@
         <v>173</v>
       </c>
       <c r="E392" s="11" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F392" t="s">
         <v>267</v>
@@ -42551,7 +42551,7 @@
         <v>173</v>
       </c>
       <c r="E399" s="11" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F399" t="s">
         <v>267</v>
@@ -42753,7 +42753,7 @@
         <v>267</v>
       </c>
       <c r="C401" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D401" t="s">
         <v>156</v>
@@ -42771,7 +42771,7 @@
         <v>46531</v>
       </c>
       <c r="I401" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J401" t="s">
         <v>267</v>
@@ -42979,7 +42979,7 @@
         <v>46498</v>
       </c>
       <c r="I403" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J403" t="s">
         <v>267</v>
@@ -43395,7 +43395,7 @@
         <v>267</v>
       </c>
       <c r="I407" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J407" s="7">
         <v>89.44</v>
@@ -43475,7 +43475,7 @@
     </row>
     <row r="408" spans="1:34" ht="12.75" customHeight="1">
       <c r="A408" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B408" t="s">
         <v>285</v>
@@ -43499,7 +43499,7 @@
         <v>267</v>
       </c>
       <c r="I408" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J408" s="7">
         <v>19.22</v>
@@ -43603,7 +43603,7 @@
         <v>51936</v>
       </c>
       <c r="I409" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J409" s="7">
         <v>12.5</v>
@@ -43695,7 +43695,7 @@
         <v>417</v>
       </c>
       <c r="E410" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F410" t="s">
         <v>267</v>
@@ -44209,7 +44209,7 @@
         <v>267</v>
       </c>
       <c r="C415" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D415" t="s">
         <v>251</v>
@@ -44227,7 +44227,7 @@
         <v>46255</v>
       </c>
       <c r="I415" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J415" s="7">
         <v>3</v>
@@ -44319,7 +44319,7 @@
         <v>251</v>
       </c>
       <c r="E416" s="11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F416" t="s">
         <v>267</v>
@@ -44420,13 +44420,13 @@
         <v>89</v>
       </c>
       <c r="D417" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E417" s="9" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="F417" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G417" s="10">
         <v>45898</v>
@@ -44435,7 +44435,7 @@
         <v>46503</v>
       </c>
       <c r="I417" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J417" t="s">
         <v>267</v>
@@ -44524,7 +44524,7 @@
         <v>267</v>
       </c>
       <c r="D418" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E418" s="11" t="s">
         <v>190</v>
@@ -44628,7 +44628,7 @@
         <v>267</v>
       </c>
       <c r="D419" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E419" s="11" t="s">
         <v>170</v>
@@ -44732,7 +44732,7 @@
         <v>267</v>
       </c>
       <c r="D420" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E420" s="11" t="s">
         <v>265</v>
@@ -44836,7 +44836,7 @@
         <v>267</v>
       </c>
       <c r="D421" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E421" s="11" t="s">
         <v>150</v>
@@ -44940,7 +44940,7 @@
         <v>267</v>
       </c>
       <c r="D422" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E422" s="11" t="s">
         <v>339</v>
@@ -45044,7 +45044,7 @@
         <v>267</v>
       </c>
       <c r="D423" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E423" s="11" t="s">
         <v>401</v>
@@ -45148,7 +45148,7 @@
         <v>267</v>
       </c>
       <c r="D424" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E424" s="11" t="s">
         <v>29</v>
@@ -45249,7 +45249,7 @@
         <v>267</v>
       </c>
       <c r="C425" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D425" t="s">
         <v>24</v>
@@ -45258,7 +45258,7 @@
         <v>24</v>
       </c>
       <c r="F425" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G425" s="10">
         <v>46114</v>
@@ -45267,7 +45267,7 @@
         <v>46283</v>
       </c>
       <c r="I425" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J425" s="7">
         <v>2.22</v>
@@ -45466,7 +45466,7 @@
         <v>76</v>
       </c>
       <c r="F427" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="G427" s="10">
         <v>46209</v>
@@ -45475,7 +45475,7 @@
         <v>46472</v>
       </c>
       <c r="I427" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J427" s="7">
         <v>1.5</v>
@@ -45671,7 +45671,7 @@
         <v>267</v>
       </c>
       <c r="E429" s="8" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F429" t="s">
         <v>267</v>
@@ -45683,7 +45683,7 @@
         <v>267</v>
       </c>
       <c r="I429" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J429" s="7">
         <v>32.72</v>
@@ -45787,7 +45787,7 @@
         <v>51936</v>
       </c>
       <c r="I430" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J430" s="7">
         <v>7.5</v>
@@ -45879,7 +45879,7 @@
         <v>417</v>
       </c>
       <c r="E431" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F431" t="s">
         <v>267</v>
@@ -46393,7 +46393,7 @@
         <v>267</v>
       </c>
       <c r="C436" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D436" t="s">
         <v>251</v>
@@ -46411,7 +46411,7 @@
         <v>46255</v>
       </c>
       <c r="I436" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J436" s="7">
         <v>15</v>
@@ -46503,7 +46503,7 @@
         <v>251</v>
       </c>
       <c r="E437" s="11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F437" t="s">
         <v>267</v>
@@ -46604,13 +46604,13 @@
         <v>89</v>
       </c>
       <c r="D438" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E438" s="9" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="F438" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G438" s="10">
         <v>45898</v>
@@ -46619,7 +46619,7 @@
         <v>46503</v>
       </c>
       <c r="I438" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J438" t="s">
         <v>267</v>
@@ -46708,7 +46708,7 @@
         <v>267</v>
       </c>
       <c r="D439" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E439" s="11" t="s">
         <v>190</v>
@@ -46812,10 +46812,10 @@
         <v>267</v>
       </c>
       <c r="D440" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E440" s="11" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F440" t="s">
         <v>267</v>
@@ -46916,7 +46916,7 @@
         <v>267</v>
       </c>
       <c r="D441" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E441" s="11" t="s">
         <v>425</v>
@@ -47020,10 +47020,10 @@
         <v>267</v>
       </c>
       <c r="D442" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E442" s="11" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F442" t="s">
         <v>267</v>
@@ -47124,7 +47124,7 @@
         <v>267</v>
       </c>
       <c r="D443" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E443" s="11" t="s">
         <v>53</v>
@@ -47228,7 +47228,7 @@
         <v>267</v>
       </c>
       <c r="D444" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E444" s="11" t="s">
         <v>349</v>
@@ -47332,7 +47332,7 @@
         <v>267</v>
       </c>
       <c r="D445" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E445" s="11" t="s">
         <v>170</v>
@@ -47436,7 +47436,7 @@
         <v>267</v>
       </c>
       <c r="D446" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E446" s="11" t="s">
         <v>6</v>
@@ -47540,7 +47540,7 @@
         <v>267</v>
       </c>
       <c r="D447" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E447" s="11" t="s">
         <v>376</v>
@@ -47644,7 +47644,7 @@
         <v>267</v>
       </c>
       <c r="D448" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E448" s="11" t="s">
         <v>265</v>
@@ -47748,7 +47748,7 @@
         <v>267</v>
       </c>
       <c r="D449" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E449" s="11" t="s">
         <v>150</v>
@@ -47852,7 +47852,7 @@
         <v>267</v>
       </c>
       <c r="D450" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E450" s="11" t="s">
         <v>339</v>
@@ -47956,7 +47956,7 @@
         <v>267</v>
       </c>
       <c r="D451" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E451" s="11" t="s">
         <v>401</v>
@@ -48060,7 +48060,7 @@
         <v>267</v>
       </c>
       <c r="D452" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E452" s="11" t="s">
         <v>29</v>
@@ -48179,7 +48179,7 @@
         <v>46514</v>
       </c>
       <c r="I453" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J453" t="s">
         <v>267</v>
@@ -48369,7 +48369,7 @@
         <v>267</v>
       </c>
       <c r="C455" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D455" t="s">
         <v>24</v>
@@ -48378,7 +48378,7 @@
         <v>24</v>
       </c>
       <c r="F455" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G455" s="10">
         <v>46114</v>
@@ -48387,7 +48387,7 @@
         <v>46283</v>
       </c>
       <c r="I455" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J455" s="7">
         <v>10.22</v>
@@ -48699,7 +48699,7 @@
         <v>267</v>
       </c>
       <c r="I458" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J458" s="7">
         <v>37.5</v>
@@ -48803,7 +48803,7 @@
         <v>51936</v>
       </c>
       <c r="I459" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J459" s="7">
         <v>37.5</v>
@@ -48895,7 +48895,7 @@
         <v>417</v>
       </c>
       <c r="E460" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F460" t="s">
         <v>267</v>
@@ -49427,7 +49427,7 @@
         <v>46304</v>
       </c>
       <c r="I465" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J465" t="s">
         <v>267</v>
@@ -49519,7 +49519,7 @@
         <v>86</v>
       </c>
       <c r="E466" s="11" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F466" t="s">
         <v>267</v>
@@ -49620,13 +49620,13 @@
         <v>89</v>
       </c>
       <c r="D467" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E467" s="9" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="F467" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G467" s="10">
         <v>45898</v>
@@ -49635,7 +49635,7 @@
         <v>46503</v>
       </c>
       <c r="I467" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J467" t="s">
         <v>267</v>
@@ -49724,7 +49724,7 @@
         <v>267</v>
       </c>
       <c r="D468" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E468" s="11" t="s">
         <v>190</v>
@@ -49828,7 +49828,7 @@
         <v>267</v>
       </c>
       <c r="D469" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E469" s="11" t="s">
         <v>366</v>
@@ -49932,7 +49932,7 @@
         <v>267</v>
       </c>
       <c r="D470" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E470" s="11" t="s">
         <v>363</v>
@@ -50036,10 +50036,10 @@
         <v>267</v>
       </c>
       <c r="D471" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E471" s="11" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F471" t="s">
         <v>267</v>
@@ -50140,7 +50140,7 @@
         <v>267</v>
       </c>
       <c r="D472" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E472" s="11" t="s">
         <v>425</v>
@@ -50244,10 +50244,10 @@
         <v>267</v>
       </c>
       <c r="D473" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E473" s="11" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F473" t="s">
         <v>267</v>
@@ -50348,7 +50348,7 @@
         <v>267</v>
       </c>
       <c r="D474" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E474" s="11" t="s">
         <v>53</v>
@@ -50452,7 +50452,7 @@
         <v>267</v>
       </c>
       <c r="D475" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E475" s="11" t="s">
         <v>349</v>
@@ -50556,7 +50556,7 @@
         <v>267</v>
       </c>
       <c r="D476" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E476" s="11" t="s">
         <v>170</v>
@@ -50660,7 +50660,7 @@
         <v>267</v>
       </c>
       <c r="D477" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E477" s="11" t="s">
         <v>6</v>
@@ -50764,7 +50764,7 @@
         <v>267</v>
       </c>
       <c r="D478" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E478" s="11" t="s">
         <v>376</v>
@@ -50868,7 +50868,7 @@
         <v>267</v>
       </c>
       <c r="D479" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E479" s="11" t="s">
         <v>265</v>
@@ -50972,7 +50972,7 @@
         <v>267</v>
       </c>
       <c r="D480" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E480" s="11" t="s">
         <v>150</v>
@@ -51076,7 +51076,7 @@
         <v>267</v>
       </c>
       <c r="D481" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E481" s="11" t="s">
         <v>339</v>
@@ -51180,7 +51180,7 @@
         <v>267</v>
       </c>
       <c r="D482" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E482" s="11" t="s">
         <v>401</v>
@@ -51284,7 +51284,7 @@
         <v>267</v>
       </c>
       <c r="D483" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E483" s="11" t="s">
         <v>29</v>
@@ -51403,7 +51403,7 @@
         <v>46514</v>
       </c>
       <c r="I484" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J484" t="s">
         <v>267</v>
@@ -52431,7 +52431,7 @@
         <v>274</v>
       </c>
       <c r="E494" s="11" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F494" t="s">
         <v>267</v>
@@ -52847,7 +52847,7 @@
         <v>274</v>
       </c>
       <c r="E498" s="11" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="F498" t="s">
         <v>267</v>
@@ -53159,7 +53159,7 @@
         <v>274</v>
       </c>
       <c r="E501" s="11" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="F501" t="s">
         <v>267</v>
@@ -53367,7 +53367,7 @@
         <v>274</v>
       </c>
       <c r="E503" s="11" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F503" t="s">
         <v>267</v>
@@ -53991,7 +53991,7 @@
         <v>274</v>
       </c>
       <c r="E509" s="11" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="F509" t="s">
         <v>267</v>
@@ -54303,7 +54303,7 @@
         <v>274</v>
       </c>
       <c r="E512" s="11" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="F512" t="s">
         <v>267</v>
@@ -54511,7 +54511,7 @@
         <v>274</v>
       </c>
       <c r="E514" s="11" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F514" t="s">
         <v>267</v>
@@ -54719,7 +54719,7 @@
         <v>274</v>
       </c>
       <c r="E516" s="11" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F516" t="s">
         <v>267</v>
@@ -54927,7 +54927,7 @@
         <v>274</v>
       </c>
       <c r="E518" s="11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F518" t="s">
         <v>267</v>
@@ -57527,7 +57527,7 @@
         <v>274</v>
       </c>
       <c r="E543" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F543" t="s">
         <v>267</v>
@@ -57625,7 +57625,7 @@
         <v>267</v>
       </c>
       <c r="C544" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D544" t="s">
         <v>24</v>
@@ -57634,7 +57634,7 @@
         <v>24</v>
       </c>
       <c r="F544" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G544" s="10">
         <v>46114</v>
@@ -57643,7 +57643,7 @@
         <v>46283</v>
       </c>
       <c r="I544" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J544" t="s">
         <v>267</v>
@@ -57851,7 +57851,7 @@
         <v>46297</v>
       </c>
       <c r="I546" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J546" t="s">
         <v>267</v>
@@ -58255,7 +58255,7 @@
         <v>429</v>
       </c>
       <c r="E550" s="11" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F550" t="s">
         <v>267</v>
@@ -58475,7 +58475,7 @@
         <v>267</v>
       </c>
       <c r="I552" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J552" s="6">
         <v>155.57</v>
@@ -58579,7 +58579,7 @@
         <v>267</v>
       </c>
       <c r="I553" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J553" s="7">
         <v>29.17</v>
@@ -58683,7 +58683,7 @@
         <v>51936</v>
       </c>
       <c r="I554" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J554" s="7">
         <v>15</v>
@@ -58775,7 +58775,7 @@
         <v>417</v>
       </c>
       <c r="E555" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F555" t="s">
         <v>267</v>
@@ -59307,7 +59307,7 @@
         <v>46315</v>
       </c>
       <c r="I560" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J560" s="7">
         <v>4</v>
@@ -59497,7 +59497,7 @@
         <v>267</v>
       </c>
       <c r="C562" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D562" t="s">
         <v>173</v>
@@ -59515,7 +59515,7 @@
         <v>47079</v>
       </c>
       <c r="I562" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J562" s="7">
         <v>6</v>
@@ -60139,7 +60139,7 @@
         <v>46454</v>
       </c>
       <c r="I568" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J568" s="7">
         <v>4.17</v>
@@ -60763,7 +60763,7 @@
         <v>46498</v>
       </c>
       <c r="I574" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J574" t="s">
         <v>267</v>
@@ -61179,7 +61179,7 @@
         <v>267</v>
       </c>
       <c r="I578" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J578" s="7">
         <v>30.75</v>
@@ -61283,7 +61283,7 @@
         <v>51936</v>
       </c>
       <c r="I579" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J579" s="7">
         <v>15</v>
@@ -61375,7 +61375,7 @@
         <v>417</v>
       </c>
       <c r="E580" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F580" t="s">
         <v>267</v>
@@ -61907,7 +61907,7 @@
         <v>46387</v>
       </c>
       <c r="I585" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J585" t="s">
         <v>267</v>
@@ -62100,10 +62100,10 @@
         <v>258</v>
       </c>
       <c r="D587" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E587" s="9" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F587" t="s">
         <v>267</v>
@@ -62115,7 +62115,7 @@
         <v>46387</v>
       </c>
       <c r="I587" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J587" t="s">
         <v>267</v>
@@ -62204,7 +62204,7 @@
         <v>267</v>
       </c>
       <c r="D588" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E588" s="11" t="s">
         <v>71</v>
@@ -62305,7 +62305,7 @@
         <v>267</v>
       </c>
       <c r="C589" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D589" t="s">
         <v>395</v>
@@ -62323,7 +62323,7 @@
         <v>46387</v>
       </c>
       <c r="I589" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J589" t="s">
         <v>267</v>
@@ -62522,7 +62522,7 @@
         <v>18</v>
       </c>
       <c r="F591" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G591" s="10">
         <v>44040</v>
@@ -62531,7 +62531,7 @@
         <v>45443</v>
       </c>
       <c r="I591" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J591" t="s">
         <v>267</v>
@@ -62721,7 +62721,7 @@
         <v>267</v>
       </c>
       <c r="C593" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D593" t="s">
         <v>20</v>
@@ -62739,7 +62739,7 @@
         <v>46022</v>
       </c>
       <c r="I593" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J593" t="s">
         <v>267</v>
@@ -62929,7 +62929,7 @@
         <v>267</v>
       </c>
       <c r="C595" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D595" t="s">
         <v>268</v>
@@ -62947,7 +62947,7 @@
         <v>46387</v>
       </c>
       <c r="I595" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J595" s="5" t="s">
         <v>267</v>
@@ -63155,7 +63155,7 @@
         <v>46387</v>
       </c>
       <c r="I597" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J597" t="s">
         <v>267</v>
@@ -63345,7 +63345,7 @@
         <v>267</v>
       </c>
       <c r="C599" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D599" t="s">
         <v>405</v>
@@ -63363,7 +63363,7 @@
         <v>46387</v>
       </c>
       <c r="I599" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J599" t="s">
         <v>267</v>
@@ -63571,7 +63571,7 @@
         <v>46416</v>
       </c>
       <c r="I601" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J601" s="7">
         <v>0.18</v>
@@ -64287,7 +64287,7 @@
         <v>46</v>
       </c>
       <c r="E608" s="11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F608" t="s">
         <v>267</v>
@@ -64388,10 +64388,10 @@
         <v>113</v>
       </c>
       <c r="D609" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E609" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F609" t="s">
         <v>267</v>
@@ -64403,7 +64403,7 @@
         <v>47003</v>
       </c>
       <c r="I609" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J609" t="s">
         <v>267</v>
@@ -64492,7 +64492,7 @@
         <v>267</v>
       </c>
       <c r="D610" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E610" s="11" t="s">
         <v>71</v>
@@ -64611,7 +64611,7 @@
         <v>47003</v>
       </c>
       <c r="I611" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J611" t="s">
         <v>267</v>
@@ -64801,7 +64801,7 @@
         <v>267</v>
       </c>
       <c r="C613" t="s">
-        <v>368</v>
+        <v>198</v>
       </c>
       <c r="D613" t="s">
         <v>107</v>
@@ -64819,7 +64819,7 @@
         <v>46387</v>
       </c>
       <c r="I613" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J613" t="s">
         <v>267</v>
@@ -65027,7 +65027,7 @@
         <v>46387</v>
       </c>
       <c r="I615" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J615" t="s">
         <v>267</v>
@@ -65217,7 +65217,7 @@
         <v>267</v>
       </c>
       <c r="C617" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D617" t="s">
         <v>381</v>
@@ -65235,7 +65235,7 @@
         <v>46387</v>
       </c>
       <c r="I617" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J617" t="s">
         <v>267</v>
@@ -65425,13 +65425,13 @@
         <v>267</v>
       </c>
       <c r="C619" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D619" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E619" s="9" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F619" t="s">
         <v>267</v>
@@ -65443,7 +65443,7 @@
         <v>46387</v>
       </c>
       <c r="I619" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J619" s="5" t="s">
         <v>267</v>
@@ -65532,7 +65532,7 @@
         <v>267</v>
       </c>
       <c r="D620" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E620" s="11" t="s">
         <v>71</v>
@@ -65633,7 +65633,7 @@
         <v>267</v>
       </c>
       <c r="C621" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D621" t="s">
         <v>95</v>
@@ -65642,7 +65642,7 @@
         <v>95</v>
       </c>
       <c r="F621" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G621" s="10">
         <v>46055</v>
@@ -65651,7 +65651,7 @@
         <v>46387</v>
       </c>
       <c r="I621" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J621" t="s">
         <v>267</v>
@@ -65841,7 +65841,7 @@
         <v>267</v>
       </c>
       <c r="C623" t="s">
-        <v>368</v>
+        <v>198</v>
       </c>
       <c r="D623" t="s">
         <v>406</v>
@@ -65859,7 +65859,7 @@
         <v>46290</v>
       </c>
       <c r="I623" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J623" s="7">
         <v>0.58</v>
@@ -66067,7 +66067,7 @@
         <v>46498</v>
       </c>
       <c r="I625" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J625" t="s">
         <v>267</v>
@@ -66275,7 +66275,7 @@
         <v>46387</v>
       </c>
       <c r="I627" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J627" s="7">
         <v>15</v>
@@ -66462,7 +66462,7 @@
         <v>74</v>
       </c>
       <c r="B629" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C629" t="s">
         <v>267</v>
@@ -66483,7 +66483,7 @@
         <v>267</v>
       </c>
       <c r="I629" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J629" s="7">
         <v>5.83</v>
@@ -66587,7 +66587,7 @@
         <v>51936</v>
       </c>
       <c r="I630" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J630" s="5" t="s">
         <v>267</v>
@@ -66679,7 +66679,7 @@
         <v>417</v>
       </c>
       <c r="E631" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F631" t="s">
         <v>267</v>
@@ -67107,7 +67107,7 @@
         <v>46259</v>
       </c>
       <c r="I635" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J635" s="7">
         <v>3</v>
@@ -67315,7 +67315,7 @@
         <v>46454</v>
       </c>
       <c r="I637" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J637" s="7">
         <v>2.83</v>
@@ -67835,7 +67835,7 @@
         <v>267</v>
       </c>
       <c r="I642" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J642" s="7">
         <v>31.08</v>
@@ -67939,7 +67939,7 @@
         <v>51936</v>
       </c>
       <c r="I643" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J643" s="7">
         <v>7.5</v>
@@ -68031,7 +68031,7 @@
         <v>417</v>
       </c>
       <c r="E644" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F644" t="s">
         <v>267</v>
@@ -68563,7 +68563,7 @@
         <v>46387</v>
       </c>
       <c r="I649" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J649" t="s">
         <v>267</v>
@@ -68756,10 +68756,10 @@
         <v>258</v>
       </c>
       <c r="D651" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E651" s="9" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F651" t="s">
         <v>267</v>
@@ -68771,7 +68771,7 @@
         <v>46387</v>
       </c>
       <c r="I651" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J651" t="s">
         <v>267</v>
@@ -68860,7 +68860,7 @@
         <v>267</v>
       </c>
       <c r="D652" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E652" s="11" t="s">
         <v>71</v>
@@ -68961,7 +68961,7 @@
         <v>267</v>
       </c>
       <c r="C653" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D653" t="s">
         <v>395</v>
@@ -68979,7 +68979,7 @@
         <v>46387</v>
       </c>
       <c r="I653" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J653" t="s">
         <v>267</v>
@@ -69178,7 +69178,7 @@
         <v>18</v>
       </c>
       <c r="F655" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G655" s="10">
         <v>44040</v>
@@ -69187,7 +69187,7 @@
         <v>45443</v>
       </c>
       <c r="I655" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J655" t="s">
         <v>267</v>
@@ -69377,7 +69377,7 @@
         <v>267</v>
       </c>
       <c r="C657" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D657" t="s">
         <v>20</v>
@@ -69395,7 +69395,7 @@
         <v>46022</v>
       </c>
       <c r="I657" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J657" t="s">
         <v>267</v>
@@ -69585,7 +69585,7 @@
         <v>267</v>
       </c>
       <c r="C659" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D659" t="s">
         <v>268</v>
@@ -69603,7 +69603,7 @@
         <v>46387</v>
       </c>
       <c r="I659" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J659" s="5" t="s">
         <v>267</v>
@@ -69811,7 +69811,7 @@
         <v>46387</v>
       </c>
       <c r="I661" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J661" t="s">
         <v>267</v>
@@ -70001,7 +70001,7 @@
         <v>267</v>
       </c>
       <c r="C663" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D663" t="s">
         <v>405</v>
@@ -70019,7 +70019,7 @@
         <v>46387</v>
       </c>
       <c r="I663" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J663" t="s">
         <v>267</v>
@@ -70209,7 +70209,7 @@
         <v>267</v>
       </c>
       <c r="C665" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D665" t="s">
         <v>171</v>
@@ -70227,7 +70227,7 @@
         <v>46493</v>
       </c>
       <c r="I665" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J665" t="s">
         <v>267</v>
@@ -70417,7 +70417,7 @@
         <v>267</v>
       </c>
       <c r="C667" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D667" t="s">
         <v>173</v>
@@ -70435,7 +70435,7 @@
         <v>47079</v>
       </c>
       <c r="I667" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J667" s="7">
         <v>1</v>
@@ -70527,7 +70527,7 @@
         <v>173</v>
       </c>
       <c r="E668" s="11" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F668" t="s">
         <v>267</v>
@@ -70747,7 +70747,7 @@
         <v>46454</v>
       </c>
       <c r="I670" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J670" t="s">
         <v>267</v>
@@ -70943,7 +70943,7 @@
         <v>176</v>
       </c>
       <c r="E672" s="11" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F672" t="s">
         <v>267</v>
@@ -71044,10 +71044,10 @@
         <v>113</v>
       </c>
       <c r="D673" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E673" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F673" t="s">
         <v>267</v>
@@ -71059,7 +71059,7 @@
         <v>47003</v>
       </c>
       <c r="I673" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J673" t="s">
         <v>267</v>
@@ -71148,7 +71148,7 @@
         <v>267</v>
       </c>
       <c r="D674" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E674" s="11" t="s">
         <v>71</v>
@@ -71267,7 +71267,7 @@
         <v>47003</v>
       </c>
       <c r="I675" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J675" t="s">
         <v>267</v>
@@ -71457,7 +71457,7 @@
         <v>267</v>
       </c>
       <c r="C677" t="s">
-        <v>368</v>
+        <v>198</v>
       </c>
       <c r="D677" t="s">
         <v>107</v>
@@ -71475,7 +71475,7 @@
         <v>46387</v>
       </c>
       <c r="I677" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J677" t="s">
         <v>267</v>
@@ -71683,7 +71683,7 @@
         <v>46387</v>
       </c>
       <c r="I679" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J679" t="s">
         <v>267</v>
@@ -71873,7 +71873,7 @@
         <v>267</v>
       </c>
       <c r="C681" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D681" t="s">
         <v>381</v>
@@ -71891,7 +71891,7 @@
         <v>46387</v>
       </c>
       <c r="I681" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J681" t="s">
         <v>267</v>
@@ -72081,13 +72081,13 @@
         <v>267</v>
       </c>
       <c r="C683" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D683" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E683" s="9" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F683" t="s">
         <v>267</v>
@@ -72099,7 +72099,7 @@
         <v>46387</v>
       </c>
       <c r="I683" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J683" s="7">
         <v>22.5</v>
@@ -72188,7 +72188,7 @@
         <v>267</v>
       </c>
       <c r="D684" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E684" s="11" t="s">
         <v>71</v>
@@ -72289,7 +72289,7 @@
         <v>267</v>
       </c>
       <c r="C685" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D685" t="s">
         <v>95</v>
@@ -72298,7 +72298,7 @@
         <v>95</v>
       </c>
       <c r="F685" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G685" s="10">
         <v>46055</v>
@@ -72307,7 +72307,7 @@
         <v>46387</v>
       </c>
       <c r="I685" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J685" t="s">
         <v>267</v>
@@ -72515,7 +72515,7 @@
         <v>46387</v>
       </c>
       <c r="I687" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J687" s="7">
         <v>0.08</v>
@@ -72702,7 +72702,7 @@
         <v>294</v>
       </c>
       <c r="B689" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C689" t="s">
         <v>267</v>
@@ -72723,7 +72723,7 @@
         <v>267</v>
       </c>
       <c r="I689" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J689" s="7">
         <v>21.08</v>
@@ -72827,7 +72827,7 @@
         <v>51936</v>
       </c>
       <c r="I690" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J690" s="7">
         <v>10</v>
@@ -72919,7 +72919,7 @@
         <v>417</v>
       </c>
       <c r="E691" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F691" t="s">
         <v>267</v>
@@ -73451,7 +73451,7 @@
         <v>46387</v>
       </c>
       <c r="I696" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J696" t="s">
         <v>267</v>
@@ -73644,10 +73644,10 @@
         <v>258</v>
       </c>
       <c r="D698" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E698" s="9" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F698" t="s">
         <v>267</v>
@@ -73659,7 +73659,7 @@
         <v>46387</v>
       </c>
       <c r="I698" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J698" t="s">
         <v>267</v>
@@ -73748,7 +73748,7 @@
         <v>267</v>
       </c>
       <c r="D699" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E699" s="11" t="s">
         <v>71</v>
@@ -73849,7 +73849,7 @@
         <v>267</v>
       </c>
       <c r="C700" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D700" t="s">
         <v>395</v>
@@ -73867,7 +73867,7 @@
         <v>46387</v>
       </c>
       <c r="I700" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J700" t="s">
         <v>267</v>
@@ -74066,7 +74066,7 @@
         <v>18</v>
       </c>
       <c r="F702" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G702" s="10">
         <v>44040</v>
@@ -74075,7 +74075,7 @@
         <v>45443</v>
       </c>
       <c r="I702" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J702" t="s">
         <v>267</v>
@@ -74265,7 +74265,7 @@
         <v>267</v>
       </c>
       <c r="C704" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D704" t="s">
         <v>20</v>
@@ -74283,7 +74283,7 @@
         <v>46022</v>
       </c>
       <c r="I704" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J704" t="s">
         <v>267</v>
@@ -74473,7 +74473,7 @@
         <v>267</v>
       </c>
       <c r="C706" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D706" t="s">
         <v>268</v>
@@ -74491,7 +74491,7 @@
         <v>46387</v>
       </c>
       <c r="I706" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J706" t="s">
         <v>267</v>
@@ -74699,7 +74699,7 @@
         <v>46387</v>
       </c>
       <c r="I708" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J708" t="s">
         <v>267</v>
@@ -74889,7 +74889,7 @@
         <v>267</v>
       </c>
       <c r="C710" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D710" t="s">
         <v>405</v>
@@ -74907,7 +74907,7 @@
         <v>46387</v>
       </c>
       <c r="I710" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J710" t="s">
         <v>267</v>
@@ -75097,7 +75097,7 @@
         <v>267</v>
       </c>
       <c r="C712" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D712" t="s">
         <v>171</v>
@@ -75115,7 +75115,7 @@
         <v>46493</v>
       </c>
       <c r="I712" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J712" s="7">
         <v>1.5</v>
@@ -75831,7 +75831,7 @@
         <v>171</v>
       </c>
       <c r="E719" s="11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F719" t="s">
         <v>267</v>
@@ -75935,7 +75935,7 @@
         <v>171</v>
       </c>
       <c r="E720" s="11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F720" t="s">
         <v>267</v>
@@ -79777,7 +79777,7 @@
         <v>267</v>
       </c>
       <c r="C757" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D757" t="s">
         <v>173</v>
@@ -79795,7 +79795,7 @@
         <v>47079</v>
       </c>
       <c r="I757" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J757" s="7">
         <v>1</v>
@@ -79887,7 +79887,7 @@
         <v>173</v>
       </c>
       <c r="E758" s="11" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F758" t="s">
         <v>267</v>
@@ -80523,7 +80523,7 @@
         <v>46454</v>
       </c>
       <c r="I764" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J764" t="s">
         <v>267</v>
@@ -80921,7 +80921,7 @@
         <v>267</v>
       </c>
       <c r="C768" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D768" t="s">
         <v>156</v>
@@ -80939,7 +80939,7 @@
         <v>46531</v>
       </c>
       <c r="I768" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J768" t="s">
         <v>267</v>
@@ -81132,10 +81132,10 @@
         <v>113</v>
       </c>
       <c r="D770" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E770" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F770" t="s">
         <v>267</v>
@@ -81147,7 +81147,7 @@
         <v>47003</v>
       </c>
       <c r="I770" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J770" t="s">
         <v>267</v>
@@ -81236,7 +81236,7 @@
         <v>267</v>
       </c>
       <c r="D771" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E771" s="11" t="s">
         <v>71</v>
@@ -81355,7 +81355,7 @@
         <v>47003</v>
       </c>
       <c r="I772" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J772" t="s">
         <v>267</v>
@@ -81545,7 +81545,7 @@
         <v>267</v>
       </c>
       <c r="C774" t="s">
-        <v>368</v>
+        <v>198</v>
       </c>
       <c r="D774" t="s">
         <v>107</v>
@@ -81563,7 +81563,7 @@
         <v>46387</v>
       </c>
       <c r="I774" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J774" t="s">
         <v>267</v>
@@ -81771,7 +81771,7 @@
         <v>46387</v>
       </c>
       <c r="I776" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J776" t="s">
         <v>267</v>
@@ -81961,7 +81961,7 @@
         <v>267</v>
       </c>
       <c r="C778" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D778" t="s">
         <v>381</v>
@@ -81979,7 +81979,7 @@
         <v>46387</v>
       </c>
       <c r="I778" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J778" t="s">
         <v>267</v>
@@ -82169,13 +82169,13 @@
         <v>267</v>
       </c>
       <c r="C780" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D780" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E780" s="9" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F780" t="s">
         <v>267</v>
@@ -82187,7 +82187,7 @@
         <v>46387</v>
       </c>
       <c r="I780" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J780" s="7">
         <v>8</v>
@@ -82276,7 +82276,7 @@
         <v>267</v>
       </c>
       <c r="D781" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E781" s="11" t="s">
         <v>71</v>
@@ -82377,7 +82377,7 @@
         <v>267</v>
       </c>
       <c r="C782" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D782" t="s">
         <v>95</v>
@@ -82386,7 +82386,7 @@
         <v>95</v>
       </c>
       <c r="F782" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G782" s="10">
         <v>46055</v>
@@ -82395,7 +82395,7 @@
         <v>46387</v>
       </c>
       <c r="I782" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J782" t="s">
         <v>267</v>
@@ -82603,7 +82603,7 @@
         <v>46498</v>
       </c>
       <c r="I784" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J784" t="s">
         <v>267</v>
@@ -82915,7 +82915,7 @@
         <v>46356</v>
       </c>
       <c r="I787" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J787" s="7">
         <v>0.5</v>
@@ -83331,7 +83331,7 @@
         <v>46387</v>
       </c>
       <c r="I791" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J791" s="7">
         <v>0.08</v>
@@ -83539,7 +83539,7 @@
         <v>267</v>
       </c>
       <c r="I793" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J793" t="s">
         <v>267</v>
@@ -83643,7 +83643,7 @@
         <v>267</v>
       </c>
       <c r="I794" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J794" s="12">
         <v>37.67</v>
@@ -83747,7 +83747,7 @@
         <v>51936</v>
       </c>
       <c r="I795" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J795" s="7">
         <v>15</v>
@@ -83839,7 +83839,7 @@
         <v>417</v>
       </c>
       <c r="E796" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F796" t="s">
         <v>267</v>
@@ -84356,10 +84356,10 @@
         <v>258</v>
       </c>
       <c r="D801" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E801" s="9" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F801" t="s">
         <v>267</v>
@@ -84371,7 +84371,7 @@
         <v>46387</v>
       </c>
       <c r="I801" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J801" t="s">
         <v>267</v>
@@ -84460,7 +84460,7 @@
         <v>267</v>
       </c>
       <c r="D802" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E802" s="11" t="s">
         <v>71</v>
@@ -84561,7 +84561,7 @@
         <v>267</v>
       </c>
       <c r="C803" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D803" t="s">
         <v>395</v>
@@ -84579,7 +84579,7 @@
         <v>46387</v>
       </c>
       <c r="I803" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J803" t="s">
         <v>267</v>
@@ -84778,7 +84778,7 @@
         <v>18</v>
       </c>
       <c r="F805" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G805" s="10">
         <v>44040</v>
@@ -84787,7 +84787,7 @@
         <v>45443</v>
       </c>
       <c r="I805" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J805" t="s">
         <v>267</v>
@@ -84977,7 +84977,7 @@
         <v>267</v>
       </c>
       <c r="C807" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D807" t="s">
         <v>20</v>
@@ -84995,7 +84995,7 @@
         <v>46022</v>
       </c>
       <c r="I807" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J807" t="s">
         <v>267</v>
@@ -85185,7 +85185,7 @@
         <v>267</v>
       </c>
       <c r="C809" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D809" t="s">
         <v>268</v>
@@ -85203,7 +85203,7 @@
         <v>46387</v>
       </c>
       <c r="I809" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J809" s="5" t="s">
         <v>267</v>
@@ -85411,7 +85411,7 @@
         <v>46387</v>
       </c>
       <c r="I811" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J811" t="s">
         <v>267</v>
@@ -85601,7 +85601,7 @@
         <v>267</v>
       </c>
       <c r="C813" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D813" t="s">
         <v>405</v>
@@ -85619,7 +85619,7 @@
         <v>46387</v>
       </c>
       <c r="I813" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J813" t="s">
         <v>267</v>
@@ -85809,7 +85809,7 @@
         <v>267</v>
       </c>
       <c r="C815" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D815" t="s">
         <v>173</v>
@@ -85827,7 +85827,7 @@
         <v>47079</v>
       </c>
       <c r="I815" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J815" s="7">
         <v>0.09</v>
@@ -86020,10 +86020,10 @@
         <v>113</v>
       </c>
       <c r="D817" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E817" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F817" t="s">
         <v>267</v>
@@ -86035,7 +86035,7 @@
         <v>47003</v>
       </c>
       <c r="I817" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J817" t="s">
         <v>267</v>
@@ -86124,7 +86124,7 @@
         <v>267</v>
       </c>
       <c r="D818" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E818" s="11" t="s">
         <v>71</v>
@@ -86243,7 +86243,7 @@
         <v>47003</v>
       </c>
       <c r="I819" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J819" t="s">
         <v>267</v>
@@ -86433,7 +86433,7 @@
         <v>267</v>
       </c>
       <c r="C821" t="s">
-        <v>368</v>
+        <v>198</v>
       </c>
       <c r="D821" t="s">
         <v>107</v>
@@ -86451,7 +86451,7 @@
         <v>46387</v>
       </c>
       <c r="I821" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J821" t="s">
         <v>267</v>
@@ -86659,7 +86659,7 @@
         <v>46387</v>
       </c>
       <c r="I823" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J823" t="s">
         <v>267</v>
@@ -86849,7 +86849,7 @@
         <v>267</v>
       </c>
       <c r="C825" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D825" t="s">
         <v>381</v>
@@ -86867,7 +86867,7 @@
         <v>46387</v>
       </c>
       <c r="I825" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J825" t="s">
         <v>267</v>
@@ -87057,13 +87057,13 @@
         <v>267</v>
       </c>
       <c r="C827" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D827" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E827" s="9" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F827" t="s">
         <v>267</v>
@@ -87075,7 +87075,7 @@
         <v>46387</v>
       </c>
       <c r="I827" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J827" s="7">
         <v>22.5</v>
@@ -87164,7 +87164,7 @@
         <v>267</v>
       </c>
       <c r="D828" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E828" s="11" t="s">
         <v>71</v>
@@ -87265,7 +87265,7 @@
         <v>267</v>
       </c>
       <c r="C829" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D829" t="s">
         <v>95</v>
@@ -87274,7 +87274,7 @@
         <v>95</v>
       </c>
       <c r="F829" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G829" s="10">
         <v>46055</v>
@@ -87283,7 +87283,7 @@
         <v>46387</v>
       </c>
       <c r="I829" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J829" t="s">
         <v>267</v>
@@ -87491,7 +87491,7 @@
         <v>46387</v>
       </c>
       <c r="I831" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J831" s="7">
         <v>0.08</v>

</xml_diff>